<commit_message>
Rediseño HTML por secciones + ajuste de precision en datos Avanter enero
- HTML con 5 secciones: Resumen (KPIs + reporte mensual + ranking),
  Clientes Directos, Avanter, Analisis y Fuentes y Datos.
- Se agrega Ceoderma via Avanter enero (355 TRX): los totales ahora
  cierran exactos contra los archivos oficiales de Avanter.
- Hojas del XLSX renombradas a nombres claros.
</commit_message>
<xml_diff>
--- a/Reporte_Labos_2026.xlsx
+++ b/Reporte_Labos_2026.xlsx
@@ -7,11 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Tabla" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="ANALISI" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Hoja 2" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Hoja 1" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Hoja2" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Tabla por Cliente" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Análisis" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Parámetros" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Promedios" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="TRX por Código" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BI59"/>
+  <dimension ref="A1:BI60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -970,7 +970,7 @@
         <v>15730</v>
       </c>
       <c r="K4" s="6" t="n">
-        <v>0.01570382172917746</v>
+        <v>0.01569825812207716</v>
       </c>
       <c r="L4" s="7" t="n">
         <v>3164020</v>
@@ -1018,7 +1018,7 @@
         <v>58552</v>
       </c>
       <c r="BG4" s="6" t="n">
-        <v>0.02274180254963603</v>
+        <v>0.02273866726835021</v>
       </c>
       <c r="BH4" s="10" t="n">
         <v>13487387</v>
@@ -1080,7 +1080,7 @@
         <v>1154</v>
       </c>
       <c r="K6" s="6" t="n">
-        <v>0.001152079483501004</v>
+        <v>0.001151671320589768</v>
       </c>
       <c r="L6" s="7" t="n">
         <v>972221.92</v>
@@ -1128,7 +1128,7 @@
         <v>4603</v>
       </c>
       <c r="BG6" s="6" t="n">
-        <v>0.001787821374777542</v>
+        <v>0.001787574898145512</v>
       </c>
       <c r="BH6" s="10" t="n">
         <v>4033286.55</v>
@@ -1190,7 +1190,7 @@
         <v>2522</v>
       </c>
       <c r="K8" s="6" t="n">
-        <v>0.002517802822694568</v>
+        <v>0.002516910806349561</v>
       </c>
       <c r="L8" s="7" t="n">
         <v>1282897</v>
@@ -1238,7 +1238,7 @@
         <v>12015</v>
       </c>
       <c r="BG8" s="6" t="n">
-        <v>0.004666668220280722</v>
+        <v>0.004666024853621189</v>
       </c>
       <c r="BH8" s="10" t="n">
         <v>6167887.15</v>
@@ -1293,7 +1293,7 @@
         <v>688</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>0.0006868550126938394</v>
+        <v>0.000686611671200832</v>
       </c>
       <c r="L9" s="7" t="n">
         <v>766721.67</v>
@@ -1329,7 +1329,7 @@
         <v>2197</v>
       </c>
       <c r="BG9" s="6" t="n">
-        <v>0.0008533225201795046</v>
+        <v>0.0008532048775202457</v>
       </c>
       <c r="BH9" s="10" t="n">
         <v>2300165.01</v>
@@ -1391,7 +1391,7 @@
         <v>4196</v>
       </c>
       <c r="K11" s="6" t="n">
-        <v>0.004189016908813009</v>
+        <v>0.004187532808660887</v>
       </c>
       <c r="L11" s="7" t="n">
         <v>7099101</v>
@@ -1439,7 +1439,7 @@
         <v>16933</v>
       </c>
       <c r="BG11" s="6" t="n">
-        <v>0.00657683670195701</v>
+        <v>0.006575929991374747</v>
       </c>
       <c r="BH11" s="10" t="n">
         <v>31379293</v>
@@ -1494,7 +1494,7 @@
         <v>63271</v>
       </c>
       <c r="K12" s="6" t="n">
-        <v>0.06316570277347662</v>
+        <v>0.0631433241984707</v>
       </c>
       <c r="L12" s="7" t="n">
         <v>6443666.51</v>
@@ -1542,7 +1542,7 @@
         <v>339671</v>
       </c>
       <c r="BG12" s="6" t="n">
-        <v>0.1319294099917581</v>
+        <v>0.1319112216441417</v>
       </c>
       <c r="BH12" s="10" t="n">
         <v>34846389.1</v>
@@ -1604,7 +1604,7 @@
         <v>18127</v>
       </c>
       <c r="K14" s="6" t="n">
-        <v>0.01809683258008899</v>
+        <v>0.0180904211683975</v>
       </c>
       <c r="L14" s="7" t="n">
         <v>1730226.41</v>
@@ -1640,13 +1640,13 @@
         <v>62353</v>
       </c>
       <c r="BG14" s="6" t="n">
-        <v>0.02421812430621422</v>
+        <v>0.02421478549295397</v>
       </c>
       <c r="BH14" s="10" t="n">
         <v>5945633.78</v>
       </c>
       <c r="BI14" s="8" t="n">
-        <v>95.35441406187351</v>
+        <v>95.35441406187353</v>
       </c>
     </row>
     <row r="15">
@@ -1702,7 +1702,7 @@
         <v>6309</v>
       </c>
       <c r="K16" s="6" t="n">
-        <v>0.006298500399833477</v>
+        <v>0.006296268944194838</v>
       </c>
       <c r="L16" s="7" t="n">
         <v>1313290.74</v>
@@ -1738,7 +1738,7 @@
         <v>18368</v>
       </c>
       <c r="BG16" s="6" t="n">
-        <v>0.00713419574449574</v>
+        <v>0.007133212194033624</v>
       </c>
       <c r="BH16" s="10" t="n">
         <v>4059529.29</v>
@@ -1800,7 +1800,7 @@
         <v>22</v>
       </c>
       <c r="K18" s="6" t="n">
-        <v>2.196338703381463e-05</v>
+        <v>2.195560576514288e-05</v>
       </c>
       <c r="L18" s="7" t="n">
         <v>1628</v>
@@ -1848,7 +1848,7 @@
         <v>72</v>
       </c>
       <c r="BG18" s="6" t="n">
-        <v>2.796505300542755e-05</v>
+        <v>2.796119762469626e-05</v>
       </c>
       <c r="BH18" s="10" t="n">
         <v>5499</v>
@@ -1910,7 +1910,7 @@
         <v>769</v>
       </c>
       <c r="K20" s="6" t="n">
-        <v>0.0007677202104092478</v>
+        <v>0.0007674482196997671</v>
       </c>
       <c r="L20" s="7" t="n">
         <v>159805.2</v>
@@ -1922,7 +1922,7 @@
         <v>769</v>
       </c>
       <c r="BG20" s="6" t="n">
-        <v>0.0002986823022385248</v>
+        <v>0.0002986411246304364</v>
       </c>
       <c r="BH20" s="10" t="n">
         <v>159805.2</v>
@@ -2058,7 +2058,7 @@
         <v>252</v>
       </c>
       <c r="BG24" s="6" t="n">
-        <v>9.787768551899642e-05</v>
+        <v>9.786419168643692e-05</v>
       </c>
       <c r="BH24" s="10" t="n">
         <v>844079.51</v>
@@ -2120,7 +2120,7 @@
         <v>8166</v>
       </c>
       <c r="K26" s="6" t="n">
-        <v>0.008152409932642286</v>
+        <v>0.008149521667188945</v>
       </c>
       <c r="L26" s="7" t="n">
         <v>1073509.3</v>
@@ -2156,7 +2156,7 @@
         <v>25707</v>
       </c>
       <c r="BG26" s="6" t="n">
-        <v>0.009984689133479529</v>
+        <v>0.009983312601917595</v>
       </c>
       <c r="BH26" s="10" t="n">
         <v>3838202.49</v>
@@ -2230,7 +2230,7 @@
         <v>76676</v>
       </c>
       <c r="BG28" s="6" t="n">
-        <v>0.02978122783672449</v>
+        <v>0.02977712207043348</v>
       </c>
       <c r="BH28" s="10" t="n">
         <v>4544586.52</v>
@@ -2296,7 +2296,7 @@
         <v>147</v>
       </c>
       <c r="K30" s="6" t="n">
-        <v>0.0001467553588168523</v>
+        <v>0.0001467033657943638</v>
       </c>
       <c r="L30" s="7" t="n">
         <v>10878</v>
@@ -2332,7 +2332,7 @@
         <v>432</v>
       </c>
       <c r="BG30" s="6" t="n">
-        <v>0.0001677903180325653</v>
+        <v>0.0001677671857481776</v>
       </c>
       <c r="BH30" s="10" t="n">
         <v>34818</v>
@@ -2391,7 +2391,7 @@
         <v>91364</v>
       </c>
       <c r="K31" s="6" t="n">
-        <v>0.09121194967988364</v>
+        <v>0.09117963477847792</v>
       </c>
       <c r="L31" s="7" t="n">
         <v>6760936</v>
@@ -2427,7 +2427,7 @@
         <v>233291</v>
       </c>
       <c r="BG31" s="6" t="n">
-        <v>0.09061104417623887</v>
+        <v>0.09059855215365299</v>
       </c>
       <c r="BH31" s="10" t="n">
         <v>18540448</v>
@@ -2486,7 +2486,7 @@
         <v>453</v>
       </c>
       <c r="K32" s="6" t="n">
-        <v>0.0004522461057417285</v>
+        <v>0.0004520858823458966</v>
       </c>
       <c r="L32" s="7" t="n">
         <v>33522</v>
@@ -2522,7 +2522,7 @@
         <v>1331</v>
       </c>
       <c r="BG32" s="6" t="n">
-        <v>0.0005169650770864454</v>
+        <v>0.0005168938060898712</v>
       </c>
       <c r="BH32" s="10" t="n">
         <v>107690</v>
@@ -2581,7 +2581,7 @@
         <v>1549</v>
       </c>
       <c r="K33" s="6" t="n">
-        <v>0.001546422114335403</v>
+        <v>0.001545874242282106</v>
       </c>
       <c r="L33" s="7" t="n">
         <v>114626</v>
@@ -2617,7 +2617,7 @@
         <v>4669</v>
       </c>
       <c r="BG33" s="6" t="n">
-        <v>0.001813456006699184</v>
+        <v>0.001813205995968151</v>
       </c>
       <c r="BH33" s="10" t="n">
         <v>377483</v>
@@ -2676,7 +2676,7 @@
         <v>42157</v>
       </c>
       <c r="K34" s="6" t="n">
-        <v>0.04208684123566016</v>
+        <v>0.04207193055641493</v>
       </c>
       <c r="L34" s="7" t="n">
         <v>3119618</v>
@@ -2712,7 +2712,7 @@
         <v>101736</v>
       </c>
       <c r="BG34" s="6" t="n">
-        <v>0.03951461989666913</v>
+        <v>0.03950917224369582</v>
       </c>
       <c r="BH34" s="10" t="n">
         <v>8080870</v>
@@ -2771,7 +2771,7 @@
         <v>34587</v>
       </c>
       <c r="K35" s="6" t="n">
-        <v>0.03452943942447939</v>
+        <v>0.03451720620904531</v>
       </c>
       <c r="L35" s="7" t="n">
         <v>2559438</v>
@@ -2807,7 +2807,7 @@
         <v>88671</v>
       </c>
       <c r="BG35" s="6" t="n">
-        <v>0.03444012798672592</v>
+        <v>0.03443537992471447</v>
       </c>
       <c r="BH35" s="10" t="n">
         <v>7041841</v>
@@ -2866,7 +2866,7 @@
         <v>1991</v>
       </c>
       <c r="K36" s="6" t="n">
-        <v>0.001987686526560224</v>
+        <v>0.001986982321745431</v>
       </c>
       <c r="L36" s="7" t="n">
         <v>147334</v>
@@ -2902,7 +2902,7 @@
         <v>6054</v>
       </c>
       <c r="BG36" s="6" t="n">
-        <v>0.0023513948735397</v>
+        <v>0.002351070700276544</v>
       </c>
       <c r="BH36" s="10" t="n">
         <v>491411</v>
@@ -2961,7 +2961,7 @@
         <v>387</v>
       </c>
       <c r="K37" s="6" t="n">
-        <v>0.0003863559446402846</v>
+        <v>0.000386219065050468</v>
       </c>
       <c r="L37" s="7" t="n">
         <v>28638</v>
@@ -2997,7 +2997,7 @@
         <v>1137</v>
       </c>
       <c r="BG37" s="6" t="n">
-        <v>0.0004416147953773768</v>
+        <v>0.0004415539124899952</v>
       </c>
       <c r="BH37" s="10" t="n">
         <v>92137</v>
@@ -3056,7 +3056,7 @@
         <v>7</v>
       </c>
       <c r="K38" s="6" t="n">
-        <v>6.98835041985011e-06</v>
+        <v>6.985874561636371e-06</v>
       </c>
       <c r="L38" s="7" t="n">
         <v>518</v>
@@ -3092,7 +3092,7 @@
         <v>21</v>
       </c>
       <c r="BG38" s="6" t="n">
-        <v>8.156473793249703e-06</v>
+        <v>8.155349307203077e-06</v>
       </c>
       <c r="BH38" s="10" t="n">
         <v>1706</v>
@@ -3151,7 +3151,7 @@
         <v>554837</v>
       </c>
       <c r="K39" s="6" t="n">
-        <v>0.5539136259854822</v>
+        <v>0.5537173834506628</v>
       </c>
       <c r="L39" s="7" t="n">
         <v>41057938</v>
@@ -3187,7 +3187,7 @@
         <v>1151690</v>
       </c>
       <c r="BG39" s="6" t="n">
-        <v>0.4473204429975119</v>
+        <v>0.4472587735053672</v>
       </c>
       <c r="BH39" s="10" t="n">
         <v>90177239</v>
@@ -3246,7 +3246,7 @@
         <v>40175</v>
       </c>
       <c r="K40" s="6" t="n">
-        <v>0.04010813973106831</v>
+        <v>0.04009393007339161</v>
       </c>
       <c r="L40" s="7" t="n">
         <v>2972950</v>
@@ -3282,7 +3282,7 @@
         <v>84177</v>
       </c>
       <c r="BG40" s="6" t="n">
-        <v>0.03269464259497049</v>
+        <v>0.03269013517297302</v>
       </c>
       <c r="BH40" s="10" t="n">
         <v>6588901</v>
@@ -3341,7 +3341,7 @@
         <v>10966</v>
       </c>
       <c r="K41" s="6" t="n">
-        <v>0.01094775010058233</v>
+        <v>0.01094387149184349</v>
       </c>
       <c r="L41" s="7" t="n">
         <v>811484</v>
@@ -3377,7 +3377,7 @@
         <v>28841</v>
       </c>
       <c r="BG41" s="6" t="n">
-        <v>0.01120194574624356</v>
+        <v>0.0112004013985259</v>
       </c>
       <c r="BH41" s="10" t="n">
         <v>2322980</v>
@@ -3436,7 +3436,7 @@
         <v>4458</v>
       </c>
       <c r="K42" s="6" t="n">
-        <v>0.004450580881670256</v>
+        <v>0.004449004113682134</v>
       </c>
       <c r="L42" s="7" t="n">
         <v>329892</v>
@@ -3472,7 +3472,7 @@
         <v>13129</v>
       </c>
       <c r="BG42" s="6" t="n">
-        <v>0.005099349734836921</v>
+        <v>0.005098646716869961</v>
       </c>
       <c r="BH42" s="10" t="n">
         <v>1056362</v>
@@ -3531,7 +3531,7 @@
         <v>26534</v>
       </c>
       <c r="K43" s="6" t="n">
-        <v>0.02648984143432897</v>
+        <v>0.02648045651692278</v>
       </c>
       <c r="L43" s="7" t="n">
         <v>1963516</v>
@@ -3567,7 +3567,7 @@
         <v>82787</v>
       </c>
       <c r="BG43" s="6" t="n">
-        <v>0.03215476171056015</v>
+        <v>0.03215032871882958</v>
       </c>
       <c r="BH43" s="10" t="n">
         <v>6723484</v>
@@ -3579,17 +3579,17 @@
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>5130</t>
+          <t>5120</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Bonos Cassara</t>
+          <t>Eximia Cepage (Ceoderma) - vía Avanter</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>CASSARA</t>
+          <t>CEODERMA</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
@@ -3604,7 +3604,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>SI - DINAMICAS - BONOS</t>
+          <t>SI - ETICOS</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -3623,68 +3623,44 @@
         </is>
       </c>
       <c r="J44" s="5" t="n">
-        <v>8603</v>
+        <v>355</v>
       </c>
       <c r="K44" s="6" t="n">
-        <v>0.008588682665995785</v>
+        <v>0.0003542836384829874</v>
       </c>
       <c r="L44" s="7" t="n">
-        <v>636622</v>
+        <v>26270</v>
       </c>
       <c r="M44" s="8" t="n">
         <v>74</v>
       </c>
-      <c r="N44" s="5" t="n">
-        <v>7894</v>
-      </c>
-      <c r="O44" s="6" t="n">
-        <v>0.0102936708398587</v>
-      </c>
-      <c r="P44" s="7" t="n">
-        <v>584156</v>
-      </c>
-      <c r="Q44" s="8" t="n">
+      <c r="BF44" s="9" t="n">
+        <v>355</v>
+      </c>
+      <c r="BG44" s="6" t="n">
+        <v>0.000137864238288433</v>
+      </c>
+      <c r="BH44" s="10" t="n">
+        <v>26270</v>
+      </c>
+      <c r="BI44" s="8" t="n">
         <v>74</v>
-      </c>
-      <c r="V44" s="5" t="n">
-        <v>9823</v>
-      </c>
-      <c r="W44" s="6" t="n">
-        <v>0.01503194460384866</v>
-      </c>
-      <c r="X44" s="7" t="n">
-        <v>913539</v>
-      </c>
-      <c r="Y44" s="8" t="n">
-        <v>93</v>
-      </c>
-      <c r="BF44" s="9" t="n">
-        <v>26320</v>
-      </c>
-      <c r="BG44" s="6" t="n">
-        <v>0.01022278048753963</v>
-      </c>
-      <c r="BH44" s="10" t="n">
-        <v>2134317</v>
-      </c>
-      <c r="BI44" s="8" t="n">
-        <v>81.09107142857142</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>5140</t>
+          <t>5130</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Bonos Bagó</t>
+          <t>Bonos Cassara</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>BAGO</t>
+          <t>CASSARA</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
@@ -3718,68 +3694,68 @@
         </is>
       </c>
       <c r="J45" s="5" t="n">
-        <v>54581</v>
+        <v>8603</v>
       </c>
       <c r="K45" s="6" t="n">
-        <v>0.05449016489511983</v>
+        <v>0.0085856398362511</v>
       </c>
       <c r="L45" s="7" t="n">
-        <v>4038994</v>
+        <v>636622</v>
       </c>
       <c r="M45" s="8" t="n">
         <v>74</v>
       </c>
       <c r="N45" s="5" t="n">
-        <v>35663</v>
+        <v>7894</v>
       </c>
       <c r="O45" s="6" t="n">
-        <v>0.04650407691435024</v>
+        <v>0.0102936708398587</v>
       </c>
       <c r="P45" s="7" t="n">
-        <v>2639062</v>
+        <v>584156</v>
       </c>
       <c r="Q45" s="8" t="n">
         <v>74</v>
       </c>
       <c r="V45" s="5" t="n">
-        <v>15759</v>
+        <v>9823</v>
       </c>
       <c r="W45" s="6" t="n">
-        <v>0.02411568920004591</v>
+        <v>0.01503194460384866</v>
       </c>
       <c r="X45" s="7" t="n">
-        <v>1465587</v>
+        <v>913539</v>
       </c>
       <c r="Y45" s="8" t="n">
         <v>93</v>
       </c>
       <c r="BF45" s="9" t="n">
-        <v>106003</v>
+        <v>26320</v>
       </c>
       <c r="BG45" s="6" t="n">
-        <v>0.04117193769075467</v>
+        <v>0.01022137113169452</v>
       </c>
       <c r="BH45" s="10" t="n">
-        <v>8143643</v>
+        <v>2134317</v>
       </c>
       <c r="BI45" s="8" t="n">
-        <v>76.82464647226965</v>
+        <v>81.09107142857142</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>5150</t>
+          <t>5140</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Bonos Caviahue</t>
+          <t>Bonos Bagó</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>CAVIAHUE</t>
+          <t>BAGO</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
@@ -3813,68 +3789,68 @@
         </is>
       </c>
       <c r="J46" s="5" t="n">
-        <v>1002</v>
+        <v>54581</v>
       </c>
       <c r="K46" s="6" t="n">
-        <v>0.00100033244581283</v>
+        <v>0.05447085992123925</v>
       </c>
       <c r="L46" s="7" t="n">
-        <v>74148</v>
+        <v>4038994</v>
       </c>
       <c r="M46" s="8" t="n">
         <v>74</v>
       </c>
       <c r="N46" s="5" t="n">
-        <v>982</v>
+        <v>35663</v>
       </c>
       <c r="O46" s="6" t="n">
-        <v>0.001280514918259595</v>
+        <v>0.04650407691435024</v>
       </c>
       <c r="P46" s="7" t="n">
-        <v>72668</v>
+        <v>2639062</v>
       </c>
       <c r="Q46" s="8" t="n">
         <v>74</v>
       </c>
       <c r="V46" s="5" t="n">
-        <v>2593</v>
+        <v>15759</v>
       </c>
       <c r="W46" s="6" t="n">
-        <v>0.003968017139140747</v>
+        <v>0.02411568920004591</v>
       </c>
       <c r="X46" s="7" t="n">
-        <v>241149</v>
+        <v>1465587</v>
       </c>
       <c r="Y46" s="8" t="n">
         <v>93</v>
       </c>
       <c r="BF46" s="9" t="n">
-        <v>4577</v>
+        <v>106003</v>
       </c>
       <c r="BG46" s="6" t="n">
-        <v>0.001777722883414471</v>
+        <v>0.04116626155292608</v>
       </c>
       <c r="BH46" s="10" t="n">
-        <v>387965</v>
+        <v>8143643</v>
       </c>
       <c r="BI46" s="8" t="n">
-        <v>84.76403757920035</v>
+        <v>76.82464647226965</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>5160</t>
+          <t>5150</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Bonos By Derm</t>
+          <t>Bonos Caviahue</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>BYDERM</t>
+          <t>CAVIAHUE</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
@@ -3908,68 +3884,68 @@
         </is>
       </c>
       <c r="J47" s="5" t="n">
-        <v>5461</v>
+        <v>1002</v>
       </c>
       <c r="K47" s="6" t="n">
-        <v>0.00545191166325735</v>
+        <v>0.0009999780443942349</v>
       </c>
       <c r="L47" s="7" t="n">
-        <v>404114</v>
+        <v>74148</v>
       </c>
       <c r="M47" s="8" t="n">
         <v>74</v>
       </c>
       <c r="N47" s="5" t="n">
-        <v>5116</v>
+        <v>982</v>
       </c>
       <c r="O47" s="6" t="n">
-        <v>0.006671195847063226</v>
+        <v>0.001280514918259595</v>
       </c>
       <c r="P47" s="7" t="n">
-        <v>378584</v>
+        <v>72668</v>
       </c>
       <c r="Q47" s="8" t="n">
         <v>74</v>
       </c>
       <c r="V47" s="5" t="n">
-        <v>6100</v>
+        <v>2593</v>
       </c>
       <c r="W47" s="6" t="n">
-        <v>0.009334710585714832</v>
+        <v>0.003968017139140747</v>
       </c>
       <c r="X47" s="7" t="n">
-        <v>567300</v>
+        <v>241149</v>
       </c>
       <c r="Y47" s="8" t="n">
         <v>93</v>
       </c>
       <c r="BF47" s="9" t="n">
-        <v>16677</v>
+        <v>4577</v>
       </c>
       <c r="BG47" s="6" t="n">
-        <v>0.006477405402382157</v>
+        <v>0.001777477799003261</v>
       </c>
       <c r="BH47" s="10" t="n">
-        <v>1349998</v>
+        <v>387965</v>
       </c>
       <c r="BI47" s="8" t="n">
-        <v>80.9496911914613</v>
+        <v>84.76403757920035</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>5170</t>
+          <t>5160</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Bonos Bioderma</t>
+          <t>Bonos By Derm</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>BIODERMA</t>
+          <t>BYDERM</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
@@ -4003,68 +3979,68 @@
         </is>
       </c>
       <c r="J48" s="5" t="n">
-        <v>1129</v>
+        <v>5461</v>
       </c>
       <c r="K48" s="6" t="n">
-        <v>0.001127121089144396</v>
+        <v>0.005449980140156603</v>
       </c>
       <c r="L48" s="7" t="n">
-        <v>83546</v>
+        <v>404114</v>
       </c>
       <c r="M48" s="8" t="n">
         <v>74</v>
       </c>
       <c r="N48" s="5" t="n">
-        <v>1053</v>
+        <v>5116</v>
       </c>
       <c r="O48" s="6" t="n">
-        <v>0.001373097972431114</v>
+        <v>0.006671195847063226</v>
       </c>
       <c r="P48" s="7" t="n">
-        <v>77922</v>
+        <v>378584</v>
       </c>
       <c r="Q48" s="8" t="n">
         <v>74</v>
       </c>
       <c r="V48" s="5" t="n">
-        <v>1462</v>
+        <v>6100</v>
       </c>
       <c r="W48" s="6" t="n">
-        <v>0.002237269979723784</v>
+        <v>0.009334710585714832</v>
       </c>
       <c r="X48" s="7" t="n">
-        <v>135966</v>
+        <v>567300</v>
       </c>
       <c r="Y48" s="8" t="n">
         <v>93</v>
       </c>
       <c r="BF48" s="9" t="n">
-        <v>3644</v>
+        <v>16677</v>
       </c>
       <c r="BG48" s="6" t="n">
-        <v>0.001415342404885805</v>
+        <v>0.006476512399820272</v>
       </c>
       <c r="BH48" s="10" t="n">
-        <v>297434</v>
+        <v>1349998</v>
       </c>
       <c r="BI48" s="8" t="n">
-        <v>81.62294182217343</v>
+        <v>80.9496911914613</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>5180</t>
+          <t>5170</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Bonos Biferdil</t>
+          <t>Bonos Bioderma</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>BIFERDIL</t>
+          <t>BIODERMA</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
@@ -4094,72 +4070,72 @@
       </c>
       <c r="I49" s="4" t="inlineStr">
         <is>
-          <t>STARTUP</t>
+          <t>PRODUCTIVO</t>
         </is>
       </c>
       <c r="J49" s="5" t="n">
-        <v>10</v>
+        <v>1129</v>
       </c>
       <c r="K49" s="6" t="n">
-        <v>9.983357742643013e-06</v>
+        <v>0.001126721768583923</v>
       </c>
       <c r="L49" s="7" t="n">
-        <v>740</v>
+        <v>83546</v>
       </c>
       <c r="M49" s="8" t="n">
         <v>74</v>
       </c>
       <c r="N49" s="5" t="n">
-        <v>12</v>
+        <v>1053</v>
       </c>
       <c r="O49" s="6" t="n">
-        <v>1.564784014166511e-05</v>
+        <v>0.001373097972431114</v>
       </c>
       <c r="P49" s="7" t="n">
-        <v>888</v>
+        <v>77922</v>
       </c>
       <c r="Q49" s="8" t="n">
         <v>74</v>
       </c>
       <c r="V49" s="5" t="n">
-        <v>22</v>
+        <v>1462</v>
       </c>
       <c r="W49" s="6" t="n">
-        <v>3.366616932552891e-05</v>
+        <v>0.002237269979723784</v>
       </c>
       <c r="X49" s="7" t="n">
-        <v>2046</v>
+        <v>135966</v>
       </c>
       <c r="Y49" s="8" t="n">
         <v>93</v>
       </c>
       <c r="BF49" s="9" t="n">
-        <v>44</v>
+        <v>3644</v>
       </c>
       <c r="BG49" s="6" t="n">
-        <v>1.708975461442795e-05</v>
+        <v>0.001415147279783239</v>
       </c>
       <c r="BH49" s="10" t="n">
-        <v>3674</v>
+        <v>297434</v>
       </c>
       <c r="BI49" s="8" t="n">
-        <v>83.5</v>
+        <v>81.62294182217343</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>5190</t>
+          <t>5180</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Bonos Fresenius</t>
+          <t>Bonos Biferdil</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>FRESENIUS</t>
+          <t>BIFERDIL</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
@@ -4193,68 +4169,68 @@
         </is>
       </c>
       <c r="J50" s="5" t="n">
-        <v>47</v>
+        <v>10</v>
       </c>
       <c r="K50" s="6" t="n">
-        <v>4.692178139042217e-05</v>
+        <v>9.979820802337674e-06</v>
       </c>
       <c r="L50" s="7" t="n">
-        <v>3478</v>
+        <v>740</v>
       </c>
       <c r="M50" s="8" t="n">
         <v>74</v>
       </c>
       <c r="N50" s="5" t="n">
-        <v>38</v>
+        <v>12</v>
       </c>
       <c r="O50" s="6" t="n">
-        <v>4.955149378193952e-05</v>
+        <v>1.564784014166511e-05</v>
       </c>
       <c r="P50" s="7" t="n">
-        <v>2812</v>
+        <v>888</v>
       </c>
       <c r="Q50" s="8" t="n">
         <v>74</v>
       </c>
       <c r="V50" s="5" t="n">
-        <v>107</v>
+        <v>22</v>
       </c>
       <c r="W50" s="6" t="n">
-        <v>0.0001637400053559815</v>
+        <v>3.366616932552891e-05</v>
       </c>
       <c r="X50" s="7" t="n">
-        <v>9951</v>
+        <v>2046</v>
       </c>
       <c r="Y50" s="8" t="n">
         <v>93</v>
       </c>
       <c r="BF50" s="9" t="n">
-        <v>192</v>
+        <v>44</v>
       </c>
       <c r="BG50" s="6" t="n">
-        <v>7.457347468114013e-05</v>
+        <v>1.708739854842549e-05</v>
       </c>
       <c r="BH50" s="10" t="n">
-        <v>16241</v>
+        <v>3674</v>
       </c>
       <c r="BI50" s="8" t="n">
-        <v>84.58854166666667</v>
+        <v>83.5</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>5200</t>
+          <t>5190</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Bonos SC Johnson</t>
+          <t>Bonos Fresenius</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>SC JHONSON</t>
+          <t>FRESENIUS</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
@@ -4288,68 +4264,68 @@
         </is>
       </c>
       <c r="J51" s="5" t="n">
-        <v>16</v>
+        <v>47</v>
       </c>
       <c r="K51" s="6" t="n">
-        <v>1.597337238822882e-05</v>
+        <v>4.690515777098706e-05</v>
       </c>
       <c r="L51" s="7" t="n">
-        <v>1184</v>
+        <v>3478</v>
       </c>
       <c r="M51" s="8" t="n">
         <v>74</v>
       </c>
       <c r="N51" s="5" t="n">
-        <v>20</v>
+        <v>38</v>
       </c>
       <c r="O51" s="6" t="n">
-        <v>2.607973356944185e-05</v>
+        <v>4.955149378193952e-05</v>
       </c>
       <c r="P51" s="7" t="n">
-        <v>1480</v>
+        <v>2812</v>
       </c>
       <c r="Q51" s="8" t="n">
         <v>74</v>
       </c>
       <c r="V51" s="5" t="n">
-        <v>6</v>
+        <v>107</v>
       </c>
       <c r="W51" s="6" t="n">
-        <v>9.181682543326065e-06</v>
+        <v>0.0001637400053559815</v>
       </c>
       <c r="X51" s="7" t="n">
-        <v>558</v>
+        <v>9951</v>
       </c>
       <c r="Y51" s="8" t="n">
         <v>93</v>
       </c>
       <c r="BF51" s="9" t="n">
-        <v>42</v>
+        <v>192</v>
       </c>
       <c r="BG51" s="6" t="n">
-        <v>1.631294758649941e-05</v>
+        <v>7.456319366585669e-05</v>
       </c>
       <c r="BH51" s="10" t="n">
-        <v>3222</v>
+        <v>16241</v>
       </c>
       <c r="BI51" s="8" t="n">
-        <v>76.71428571428571</v>
+        <v>84.58854166666667</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>5210</t>
+          <t>5200</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Bonos Pharmatrix</t>
+          <t>Bonos SC Johnson</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>PHARMATRIX</t>
+          <t>SC JHONSON</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
@@ -4383,68 +4359,68 @@
         </is>
       </c>
       <c r="J52" s="5" t="n">
-        <v>85</v>
+        <v>16</v>
       </c>
       <c r="K52" s="6" t="n">
-        <v>8.485854081246562e-05</v>
+        <v>1.596771328374028e-05</v>
       </c>
       <c r="L52" s="7" t="n">
-        <v>6290</v>
+        <v>1184</v>
       </c>
       <c r="M52" s="8" t="n">
         <v>74</v>
       </c>
       <c r="N52" s="5" t="n">
-        <v>80</v>
+        <v>20</v>
       </c>
       <c r="O52" s="6" t="n">
-        <v>0.0001043189342777674</v>
+        <v>2.607973356944185e-05</v>
       </c>
       <c r="P52" s="7" t="n">
-        <v>5920</v>
+        <v>1480</v>
       </c>
       <c r="Q52" s="8" t="n">
         <v>74</v>
       </c>
       <c r="V52" s="5" t="n">
-        <v>320</v>
+        <v>6</v>
       </c>
       <c r="W52" s="6" t="n">
-        <v>0.0004896897356440568</v>
+        <v>9.181682543326065e-06</v>
       </c>
       <c r="X52" s="7" t="n">
-        <v>29760</v>
+        <v>558</v>
       </c>
       <c r="Y52" s="8" t="n">
         <v>93</v>
       </c>
       <c r="BF52" s="9" t="n">
-        <v>485</v>
+        <v>42</v>
       </c>
       <c r="BG52" s="6" t="n">
-        <v>0.0001883757042726717</v>
+        <v>1.631069861440615e-05</v>
       </c>
       <c r="BH52" s="10" t="n">
-        <v>41970</v>
+        <v>3222</v>
       </c>
       <c r="BI52" s="8" t="n">
-        <v>86.5360824742268</v>
+        <v>76.71428571428571</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>5220</t>
+          <t>5210</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Bonos Megalabs</t>
+          <t>Bonos Pharmatrix</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>MEGALABS</t>
+          <t>PHARMATRIX</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
@@ -4478,38 +4454,68 @@
         </is>
       </c>
       <c r="J53" s="5" t="n">
-        <v>0</v>
+        <v>85</v>
       </c>
       <c r="K53" s="6" t="n">
-        <v>0</v>
+        <v>8.482847681987022e-05</v>
       </c>
       <c r="L53" s="7" t="n">
-        <v>0</v>
+        <v>6290</v>
+      </c>
+      <c r="M53" s="8" t="n">
+        <v>74</v>
       </c>
       <c r="N53" s="5" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="O53" s="6" t="n">
-        <v>0</v>
+        <v>0.0001043189342777674</v>
       </c>
       <c r="P53" s="7" t="n">
-        <v>0</v>
+        <v>5920</v>
+      </c>
+      <c r="Q53" s="8" t="n">
+        <v>74</v>
+      </c>
+      <c r="V53" s="5" t="n">
+        <v>320</v>
+      </c>
+      <c r="W53" s="6" t="n">
+        <v>0.0004896897356440568</v>
+      </c>
+      <c r="X53" s="7" t="n">
+        <v>29760</v>
+      </c>
+      <c r="Y53" s="8" t="n">
+        <v>93</v>
+      </c>
+      <c r="BF53" s="9" t="n">
+        <v>485</v>
+      </c>
+      <c r="BG53" s="6" t="n">
+        <v>0.0001883497339996901</v>
+      </c>
+      <c r="BH53" s="10" t="n">
+        <v>41970</v>
+      </c>
+      <c r="BI53" s="8" t="n">
+        <v>86.5360824742268</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>5230</t>
+          <t>5220</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Bonos Siegfried</t>
+          <t>Bonos Megalabs</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>SIEGFRIED</t>
+          <t>MEGALABS</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
@@ -4551,21 +4557,30 @@
       <c r="L54" s="7" t="n">
         <v>0</v>
       </c>
+      <c r="N54" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O54" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P54" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>5240</t>
+          <t>5230</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Bonos Raisse</t>
+          <t>Bonos Siegfried</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>RAISSE</t>
+          <t>SIEGFRIED</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
@@ -4599,56 +4614,29 @@
         </is>
       </c>
       <c r="J55" s="5" t="n">
-        <v>167</v>
+        <v>0</v>
       </c>
       <c r="K55" s="6" t="n">
-        <v>0.0001667220743021383</v>
+        <v>0</v>
       </c>
       <c r="L55" s="7" t="n">
-        <v>12358</v>
-      </c>
-      <c r="M55" s="8" t="n">
-        <v>74</v>
-      </c>
-      <c r="N55" s="5" t="n">
-        <v>356</v>
-      </c>
-      <c r="O55" s="6" t="n">
-        <v>0.000464219257536065</v>
-      </c>
-      <c r="P55" s="7" t="n">
-        <v>26344</v>
-      </c>
-      <c r="Q55" s="8" t="n">
-        <v>74</v>
-      </c>
-      <c r="BF55" s="9" t="n">
-        <v>523</v>
-      </c>
-      <c r="BG55" s="6" t="n">
-        <v>0.000203135037803314</v>
-      </c>
-      <c r="BH55" s="10" t="n">
-        <v>38702</v>
-      </c>
-      <c r="BI55" s="8" t="n">
-        <v>74</v>
+        <v>0</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>5250</t>
+          <t>5240</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Bonos Siscom (Rayito de Sol)</t>
+          <t>Bonos Raisse</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>SISCOM</t>
+          <t>RAISSE</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
@@ -4682,62 +4670,56 @@
         </is>
       </c>
       <c r="J56" s="5" t="n">
-        <v>0</v>
+        <v>167</v>
       </c>
       <c r="K56" s="6" t="n">
-        <v>0</v>
+        <v>0.0001666630073990391</v>
       </c>
       <c r="L56" s="7" t="n">
-        <v>0</v>
+        <v>12358</v>
+      </c>
+      <c r="M56" s="8" t="n">
+        <v>74</v>
       </c>
       <c r="N56" s="5" t="n">
-        <v>0</v>
+        <v>356</v>
       </c>
       <c r="O56" s="6" t="n">
-        <v>0</v>
+        <v>0.000464219257536065</v>
       </c>
       <c r="P56" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="V56" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="W56" s="6" t="n">
-        <v>1.530280423887677e-06</v>
-      </c>
-      <c r="X56" s="7" t="n">
-        <v>93</v>
-      </c>
-      <c r="Y56" s="8" t="n">
-        <v>93</v>
+        <v>26344</v>
+      </c>
+      <c r="Q56" s="8" t="n">
+        <v>74</v>
       </c>
       <c r="BF56" s="9" t="n">
-        <v>1</v>
+        <v>523</v>
       </c>
       <c r="BG56" s="6" t="n">
-        <v>3.884035139642715e-07</v>
+        <v>0.0002031070327460576</v>
       </c>
       <c r="BH56" s="10" t="n">
-        <v>93</v>
+        <v>38702</v>
       </c>
       <c r="BI56" s="8" t="n">
-        <v>93</v>
+        <v>74</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>5260</t>
+          <t>5250</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Bonos ENA (alta 22/04/2026)</t>
+          <t>Bonos Siscom (Rayito de Sol)</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>ENA</t>
+          <t>SISCOM</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
@@ -4750,15 +4732,19 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="F57" t="inlineStr"/>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>SI - DINAMICAS - BONOS</t>
+        </is>
+      </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Alta laboratorio nuevo - Avanter</t>
+          <t>Facturado vía Avanter - valor unitario por TRX</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>Mensual</t>
+          <t>Trimestral por IPC Indec</t>
         </is>
       </c>
       <c r="I57" s="4" t="inlineStr">
@@ -4766,27 +4752,63 @@
           <t>STARTUP</t>
         </is>
       </c>
+      <c r="J57" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K57" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L57" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N57" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O57" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P57" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="V57" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="W57" s="6" t="n">
+        <v>1.530280423887677e-06</v>
+      </c>
       <c r="X57" s="7" t="n">
-        <v>547420.8</v>
+        <v>93</v>
+      </c>
+      <c r="Y57" s="8" t="n">
+        <v>93</v>
+      </c>
+      <c r="BF57" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="BG57" s="6" t="n">
+        <v>3.883499670096703e-07</v>
       </c>
       <c r="BH57" s="10" t="n">
-        <v>547420.8</v>
+        <v>93</v>
+      </c>
+      <c r="BI57" s="8" t="n">
+        <v>93</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>5270</t>
+          <t>5260</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Bonos Convatec (alta 24/04/2026)</t>
+          <t>Bonos ENA (alta 22/04/2026)</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>CONVATEC</t>
+          <t>ENA</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
@@ -4823,83 +4845,132 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="11" t="inlineStr">
+      <c r="A59" s="4" t="inlineStr">
+        <is>
+          <t>5270</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Bonos Convatec (alta 24/04/2026)</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>CONVATEC</t>
+        </is>
+      </c>
+      <c r="D59" s="4" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E59" s="4" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr"/>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Alta laboratorio nuevo - Avanter</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Mensual</t>
+        </is>
+      </c>
+      <c r="I59" s="4" t="inlineStr">
+        <is>
+          <t>STARTUP</t>
+        </is>
+      </c>
+      <c r="X59" s="7" t="n">
+        <v>547420.8</v>
+      </c>
+      <c r="BH59" s="10" t="n">
+        <v>547420.8</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="11" t="inlineStr">
         <is>
           <t>TOTAL GENERAL</t>
         </is>
       </c>
-      <c r="J59" s="12" t="n">
-        <v>1001667</v>
-      </c>
-      <c r="K59" s="13" t="n"/>
-      <c r="L59" s="14" t="n">
-        <v>89679849.75</v>
-      </c>
-      <c r="M59" s="13" t="n"/>
-      <c r="N59" s="12" t="n">
+      <c r="J60" s="12" t="n">
+        <v>1002022</v>
+      </c>
+      <c r="K60" s="13" t="n"/>
+      <c r="L60" s="14" t="n">
+        <v>89706119.75</v>
+      </c>
+      <c r="M60" s="13" t="n"/>
+      <c r="N60" s="12" t="n">
         <v>766879</v>
       </c>
-      <c r="O59" s="13" t="n"/>
-      <c r="P59" s="14" t="n">
+      <c r="O60" s="13" t="n"/>
+      <c r="P60" s="14" t="n">
         <v>69228656.50999999</v>
       </c>
-      <c r="Q59" s="13" t="n"/>
-      <c r="R59" s="12" t="n">
+      <c r="Q60" s="13" t="n"/>
+      <c r="R60" s="12" t="n">
         <v>152621</v>
       </c>
-      <c r="S59" s="13" t="n"/>
-      <c r="T59" s="14" t="n">
+      <c r="S60" s="13" t="n"/>
+      <c r="T60" s="14" t="n">
         <v>29259222.98</v>
       </c>
-      <c r="U59" s="13" t="n"/>
-      <c r="V59" s="12" t="n">
+      <c r="U60" s="13" t="n"/>
+      <c r="V60" s="12" t="n">
         <v>653475</v>
       </c>
-      <c r="W59" s="13" t="n"/>
-      <c r="X59" s="14" t="n">
+      <c r="W60" s="13" t="n"/>
+      <c r="X60" s="14" t="n">
         <v>80417563.47999999</v>
       </c>
-      <c r="Y59" s="13" t="n"/>
-      <c r="Z59" s="12" t="n"/>
-      <c r="AA59" s="13" t="n"/>
-      <c r="AB59" s="14" t="n"/>
-      <c r="AC59" s="13" t="n"/>
-      <c r="AD59" s="12" t="n"/>
-      <c r="AE59" s="13" t="n"/>
-      <c r="AF59" s="14" t="n"/>
-      <c r="AG59" s="13" t="n"/>
-      <c r="AH59" s="12" t="n"/>
-      <c r="AI59" s="13" t="n"/>
-      <c r="AJ59" s="14" t="n"/>
-      <c r="AK59" s="13" t="n"/>
-      <c r="AL59" s="12" t="n"/>
-      <c r="AM59" s="13" t="n"/>
-      <c r="AN59" s="14" t="n"/>
-      <c r="AO59" s="13" t="n"/>
-      <c r="AP59" s="12" t="n"/>
-      <c r="AQ59" s="13" t="n"/>
-      <c r="AR59" s="14" t="n"/>
-      <c r="AS59" s="13" t="n"/>
-      <c r="AT59" s="12" t="n"/>
-      <c r="AU59" s="13" t="n"/>
-      <c r="AV59" s="14" t="n"/>
-      <c r="AW59" s="13" t="n"/>
-      <c r="AX59" s="12" t="n"/>
-      <c r="AY59" s="13" t="n"/>
-      <c r="AZ59" s="14" t="n"/>
-      <c r="BA59" s="13" t="n"/>
-      <c r="BB59" s="12" t="n"/>
-      <c r="BC59" s="13" t="n"/>
-      <c r="BD59" s="14" t="n"/>
-      <c r="BE59" s="13" t="n"/>
-      <c r="BF59" s="12" t="n">
-        <v>2574642</v>
-      </c>
-      <c r="BG59" s="13" t="n"/>
-      <c r="BH59" s="14" t="n">
-        <v>268585292.72</v>
-      </c>
-      <c r="BI59" s="13" t="n"/>
+      <c r="Y60" s="13" t="n"/>
+      <c r="Z60" s="12" t="n"/>
+      <c r="AA60" s="13" t="n"/>
+      <c r="AB60" s="14" t="n"/>
+      <c r="AC60" s="13" t="n"/>
+      <c r="AD60" s="12" t="n"/>
+      <c r="AE60" s="13" t="n"/>
+      <c r="AF60" s="14" t="n"/>
+      <c r="AG60" s="13" t="n"/>
+      <c r="AH60" s="12" t="n"/>
+      <c r="AI60" s="13" t="n"/>
+      <c r="AJ60" s="14" t="n"/>
+      <c r="AK60" s="13" t="n"/>
+      <c r="AL60" s="12" t="n"/>
+      <c r="AM60" s="13" t="n"/>
+      <c r="AN60" s="14" t="n"/>
+      <c r="AO60" s="13" t="n"/>
+      <c r="AP60" s="12" t="n"/>
+      <c r="AQ60" s="13" t="n"/>
+      <c r="AR60" s="14" t="n"/>
+      <c r="AS60" s="13" t="n"/>
+      <c r="AT60" s="12" t="n"/>
+      <c r="AU60" s="13" t="n"/>
+      <c r="AV60" s="14" t="n"/>
+      <c r="AW60" s="13" t="n"/>
+      <c r="AX60" s="12" t="n"/>
+      <c r="AY60" s="13" t="n"/>
+      <c r="AZ60" s="14" t="n"/>
+      <c r="BA60" s="13" t="n"/>
+      <c r="BB60" s="12" t="n"/>
+      <c r="BC60" s="13" t="n"/>
+      <c r="BD60" s="14" t="n"/>
+      <c r="BE60" s="13" t="n"/>
+      <c r="BF60" s="12" t="n">
+        <v>2574997</v>
+      </c>
+      <c r="BG60" s="13" t="n"/>
+      <c r="BH60" s="14" t="n">
+        <v>268611562.72</v>
+      </c>
+      <c r="BI60" s="13" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="27">
@@ -4925,7 +4996,7 @@
     <mergeCell ref="AD1:AG1"/>
     <mergeCell ref="AP1:AS1"/>
     <mergeCell ref="AH1:AK1"/>
-    <mergeCell ref="A59:I59"/>
+    <mergeCell ref="A60:I60"/>
     <mergeCell ref="N1:Q1"/>
     <mergeCell ref="BB1:BE1"/>
     <mergeCell ref="A7:BI7"/>
@@ -5219,10 +5290,10 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>1956474</v>
+        <v>1956829</v>
       </c>
       <c r="C21" s="7" t="n">
-        <v>155149470.6</v>
+        <v>155175740.6</v>
       </c>
     </row>
   </sheetData>
@@ -5236,64 +5307,84 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>Parámetros (heredado 2025 - ajustar si cambió)</t>
+          <t>Parámetros de facturación 2026</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Descuento</t>
+          <t>VU Avanter Enero/Febrero</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>60</v>
-      </c>
-      <c r="C3" t="n">
-        <v>5</v>
-      </c>
+        <v>74</v>
+      </c>
+      <c r="C3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Set up</t>
+          <t>VU Avanter Abril</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1000000</v>
+        <v>93</v>
       </c>
       <c r="C4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Bonos</t>
+          <t>Alta lab nuevo Avanter (base dic-25)</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>150</v>
+        <v>500000</v>
       </c>
       <c r="C5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Dinámica</t>
+          <t>Alta lab nuevo Avanter (marzo, IPC acum)</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>135</v>
+        <v>547420.8</v>
       </c>
       <c r="C6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Mínimo Sidus Farma</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>766721.67</v>
+      </c>
+      <c r="C7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Mínimo Bayer (mar-abr)</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>844447.62</v>
+      </c>
+      <c r="C8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5350,7 +5441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B44"/>
+  <dimension ref="A1:B45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5365,7 +5456,7 @@
       </c>
       <c r="B1" s="16" t="inlineStr">
         <is>
-          <t>(TRX acum ene-abr)</t>
+          <t>TRX acum ene-abr</t>
         </is>
       </c>
     </row>
@@ -5682,87 +5773,87 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>5300</t>
+          <t>5120</t>
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>252</v>
+        <v>355</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>5190</t>
+          <t>5300</t>
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>192</v>
+        <v>252</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>5070</t>
+          <t>5190</t>
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>72</v>
+        <v>192</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>5180</t>
+          <t>5070</t>
         </is>
       </c>
       <c r="B36" s="5" t="n">
-        <v>44</v>
+        <v>72</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>5200</t>
+          <t>5180</t>
         </is>
       </c>
       <c r="B37" s="5" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>5027</t>
+          <t>5200</t>
         </is>
       </c>
       <c r="B38" s="5" t="n">
-        <v>21</v>
+        <v>42</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>5250</t>
+          <t>5027</t>
         </is>
       </c>
       <c r="B39" s="5" t="n">
-        <v>1</v>
+        <v>21</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>5026</t>
+          <t>5250</t>
         </is>
       </c>
       <c r="B40" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>5220</t>
+          <t>5026</t>
         </is>
       </c>
       <c r="B41" s="5" t="n">
@@ -5772,7 +5863,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>5230</t>
+          <t>5220</t>
         </is>
       </c>
       <c r="B42" s="5" t="n">
@@ -5782,7 +5873,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>5260</t>
+          <t>5230</t>
         </is>
       </c>
       <c r="B43" s="5" t="n">
@@ -5792,10 +5883,20 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
+          <t>5260</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
           <t>5270</t>
         </is>
       </c>
-      <c r="B44" s="5" t="n">
+      <c r="B45" s="5" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Incorporar Avanter marzo (532.345 TRX) y excluir Provincia ART y Serdata
- Avanter marzo desde archivo oficial: 532.345 TRX x $74 = $39.393.530.
  Los 4 meses quedan completos para Avanter.
- Provincia ART (convenio de servicios) y Serdata (proveedor) se excluyen
  del reporte de laboratorios por definicion del negocio.
- Nuevo total ene-abr: $299.622.303,70 / 3.004.959 TRX.
</commit_message>
<xml_diff>
--- a/Reporte_Labos_2026.xlsx
+++ b/Reporte_Labos_2026.xlsx
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BI60"/>
+  <dimension ref="A1:BI56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -970,7 +970,7 @@
         <v>15730</v>
       </c>
       <c r="K4" s="6" t="n">
-        <v>0.01569825812207716</v>
+        <v>0.0158272425784017</v>
       </c>
       <c r="L4" s="7" t="n">
         <v>3164020</v>
@@ -982,7 +982,7 @@
         <v>13198</v>
       </c>
       <c r="O4" s="6" t="n">
-        <v>0.01721001618247468</v>
+        <v>0.01912191051038608</v>
       </c>
       <c r="P4" s="7" t="n">
         <v>2976652</v>
@@ -994,7 +994,7 @@
         <v>14775</v>
       </c>
       <c r="S4" s="6" t="n">
-        <v>0.09680843396387129</v>
+        <v>0.02184765346590287</v>
       </c>
       <c r="T4" s="7" t="n">
         <v>3447758</v>
@@ -1006,7 +1006,7 @@
         <v>14849</v>
       </c>
       <c r="W4" s="6" t="n">
-        <v>0.02272313401430812</v>
+        <v>0.02303506219109996</v>
       </c>
       <c r="X4" s="7" t="n">
         <v>3898957</v>
@@ -1018,7 +1018,7 @@
         <v>58552</v>
       </c>
       <c r="BG4" s="6" t="n">
-        <v>0.02273866726835021</v>
+        <v>0.01948512442266267</v>
       </c>
       <c r="BH4" s="10" t="n">
         <v>13487387</v>
@@ -1080,7 +1080,7 @@
         <v>1154</v>
       </c>
       <c r="K6" s="6" t="n">
-        <v>0.001151671320589768</v>
+        <v>0.001161134007341104</v>
       </c>
       <c r="L6" s="7" t="n">
         <v>972221.92</v>
@@ -1092,7 +1092,7 @@
         <v>1090</v>
       </c>
       <c r="O6" s="6" t="n">
-        <v>0.001421345479534581</v>
+        <v>0.001579245526316171</v>
       </c>
       <c r="P6" s="7" t="n">
         <v>941267.72</v>
@@ -1104,7 +1104,7 @@
         <v>1181</v>
       </c>
       <c r="S6" s="6" t="n">
-        <v>0.007738122538838037</v>
+        <v>0.001746333586682321</v>
       </c>
       <c r="T6" s="7" t="n">
         <v>1044493.17</v>
@@ -1116,7 +1116,7 @@
         <v>1178</v>
       </c>
       <c r="W6" s="6" t="n">
-        <v>0.001802670339339684</v>
+        <v>0.001827416207227136</v>
       </c>
       <c r="X6" s="7" t="n">
         <v>1075303.74</v>
@@ -1128,7 +1128,7 @@
         <v>4603</v>
       </c>
       <c r="BG6" s="6" t="n">
-        <v>0.001787574898145512</v>
+        <v>0.001531801265840898</v>
       </c>
       <c r="BH6" s="10" t="n">
         <v>4033286.55</v>
@@ -1190,7 +1190,7 @@
         <v>2522</v>
       </c>
       <c r="K8" s="6" t="n">
-        <v>0.002516910806349561</v>
+        <v>0.002537590958851182</v>
       </c>
       <c r="L8" s="7" t="n">
         <v>1282897</v>
@@ -1202,7 +1202,7 @@
         <v>2281</v>
       </c>
       <c r="O8" s="6" t="n">
-        <v>0.002974393613594843</v>
+        <v>0.003304824812410262</v>
       </c>
       <c r="P8" s="7" t="n">
         <v>1255491</v>
@@ -1214,7 +1214,7 @@
         <v>2333</v>
       </c>
       <c r="S8" s="6" t="n">
-        <v>0.01528623190779775</v>
+        <v>0.003449785146257286</v>
       </c>
       <c r="T8" s="7" t="n">
         <v>1330813</v>
@@ -1226,7 +1226,7 @@
         <v>4879</v>
       </c>
       <c r="W8" s="6" t="n">
-        <v>0.007466238188147978</v>
+        <v>0.007568729775094396</v>
       </c>
       <c r="X8" s="7" t="n">
         <v>2298686.15</v>
@@ -1238,7 +1238,7 @@
         <v>12015</v>
       </c>
       <c r="BG8" s="6" t="n">
-        <v>0.004666024853621189</v>
+        <v>0.003998390660238625</v>
       </c>
       <c r="BH8" s="10" t="n">
         <v>6167887.15</v>
@@ -1293,7 +1293,7 @@
         <v>688</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>0.000686611671200832</v>
+        <v>0.000692253203683431</v>
       </c>
       <c r="L9" s="7" t="n">
         <v>766721.67</v>
@@ -1305,7 +1305,7 @@
         <v>615</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>0.004029589637074845</v>
+        <v>0.0009093947127939267</v>
       </c>
       <c r="T9" s="7" t="n">
         <v>766721.67</v>
@@ -1317,7 +1317,7 @@
         <v>894</v>
       </c>
       <c r="W9" s="6" t="n">
-        <v>0.001368070698955584</v>
+        <v>0.0013868506700009</v>
       </c>
       <c r="X9" s="7" t="n">
         <v>766721.67</v>
@@ -1329,7 +1329,7 @@
         <v>2197</v>
       </c>
       <c r="BG9" s="6" t="n">
-        <v>0.0008532048775202457</v>
+        <v>0.0007311247840652734</v>
       </c>
       <c r="BH9" s="10" t="n">
         <v>2300165.01</v>
@@ -1391,7 +1391,7 @@
         <v>4196</v>
       </c>
       <c r="K11" s="6" t="n">
-        <v>0.004187532808660887</v>
+        <v>0.00422193959688325</v>
       </c>
       <c r="L11" s="7" t="n">
         <v>7099101</v>
@@ -1403,7 +1403,7 @@
         <v>3565</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>0.00464871250875301</v>
+        <v>0.005165147065428577</v>
       </c>
       <c r="P11" s="7" t="n">
         <v>6836393</v>
@@ -1415,7 +1415,7 @@
         <v>4586</v>
       </c>
       <c r="S11" s="6" t="n">
-        <v>0.03004828955386218</v>
+        <v>0.006781275045321867</v>
       </c>
       <c r="T11" s="7" t="n">
         <v>8378215</v>
@@ -1427,7 +1427,7 @@
         <v>4586</v>
       </c>
       <c r="W11" s="6" t="n">
-        <v>0.007017866023948888</v>
+        <v>0.007114202653941975</v>
       </c>
       <c r="X11" s="7" t="n">
         <v>9065584</v>
@@ -1439,7 +1439,7 @@
         <v>16933</v>
       </c>
       <c r="BG11" s="6" t="n">
-        <v>0.006575929991374747</v>
+        <v>0.005635018647509001</v>
       </c>
       <c r="BH11" s="10" t="n">
         <v>31379293</v>
@@ -1494,7 +1494,7 @@
         <v>63271</v>
       </c>
       <c r="K12" s="6" t="n">
-        <v>0.0631433241984707</v>
+        <v>0.0636621401893232</v>
       </c>
       <c r="L12" s="7" t="n">
         <v>6443666.51</v>
@@ -1506,7 +1506,7 @@
         <v>82475</v>
       </c>
       <c r="O12" s="6" t="n">
-        <v>0.1075463013069859</v>
+        <v>0.1194938300760791</v>
       </c>
       <c r="P12" s="7" t="n">
         <v>8320434.77</v>
@@ -1518,7 +1518,7 @@
         <v>90524</v>
       </c>
       <c r="S12" s="6" t="n">
-        <v>0.5931293858643306</v>
+        <v>0.1338569869609064</v>
       </c>
       <c r="T12" s="7" t="n">
         <v>9289060.32</v>
@@ -1530,7 +1530,7 @@
         <v>103401</v>
       </c>
       <c r="W12" s="6" t="n">
-        <v>0.1582325261104097</v>
+        <v>0.1604046377279228</v>
       </c>
       <c r="X12" s="7" t="n">
         <v>10793227.5</v>
@@ -1542,7 +1542,7 @@
         <v>339671</v>
       </c>
       <c r="BG12" s="6" t="n">
-        <v>0.1319112216441417</v>
+        <v>0.1130368168084823</v>
       </c>
       <c r="BH12" s="10" t="n">
         <v>34846389.1</v>
@@ -1604,7 +1604,7 @@
         <v>18127</v>
       </c>
       <c r="K14" s="6" t="n">
-        <v>0.0180904211683975</v>
+        <v>0.01823906078949063</v>
       </c>
       <c r="L14" s="7" t="n">
         <v>1730226.41</v>
@@ -1616,7 +1616,7 @@
         <v>23875</v>
       </c>
       <c r="S14" s="6" t="n">
-        <v>0.1564332562360357</v>
+        <v>0.03530373783407317</v>
       </c>
       <c r="T14" s="7" t="n">
         <v>2338884.94</v>
@@ -1628,7 +1628,7 @@
         <v>20351</v>
       </c>
       <c r="W14" s="6" t="n">
-        <v>0.03114273690653812</v>
+        <v>0.03157024383130683</v>
       </c>
       <c r="X14" s="7" t="n">
         <v>1876522.43</v>
@@ -1640,7 +1640,7 @@
         <v>62353</v>
       </c>
       <c r="BG14" s="6" t="n">
-        <v>0.02421478549295397</v>
+        <v>0.02075003352791169</v>
       </c>
       <c r="BH14" s="10" t="n">
         <v>5945633.78</v>
@@ -1702,7 +1702,7 @@
         <v>6309</v>
       </c>
       <c r="K16" s="6" t="n">
-        <v>0.006296268944194838</v>
+        <v>0.006348002125056347</v>
       </c>
       <c r="L16" s="7" t="n">
         <v>1313290.74</v>
@@ -1714,7 +1714,7 @@
         <v>6019</v>
       </c>
       <c r="S16" s="6" t="n">
-        <v>0.03943756101716016</v>
+        <v>0.008900238660661211</v>
       </c>
       <c r="T16" s="7" t="n">
         <v>1368036.9</v>
@@ -1726,7 +1726,7 @@
         <v>6040</v>
       </c>
       <c r="W16" s="6" t="n">
-        <v>0.009242893760281572</v>
+        <v>0.009369774101572075</v>
       </c>
       <c r="X16" s="7" t="n">
         <v>1378201.65</v>
@@ -1738,7 +1738,7 @@
         <v>18368</v>
       </c>
       <c r="BG16" s="6" t="n">
-        <v>0.007133212194033624</v>
+        <v>0.00611256260068773</v>
       </c>
       <c r="BH16" s="10" t="n">
         <v>4059529.29</v>
@@ -1800,7 +1800,7 @@
         <v>22</v>
       </c>
       <c r="K18" s="6" t="n">
-        <v>2.195560576514288e-05</v>
+        <v>2.213600360615622e-05</v>
       </c>
       <c r="L18" s="7" t="n">
         <v>1628</v>
@@ -1812,7 +1812,7 @@
         <v>20</v>
       </c>
       <c r="O18" s="6" t="n">
-        <v>2.607973356944185e-05</v>
+        <v>2.897698213424167e-05</v>
       </c>
       <c r="P18" s="7" t="n">
         <v>1480</v>
@@ -1824,7 +1824,7 @@
         <v>21</v>
       </c>
       <c r="S18" s="6" t="n">
-        <v>0.0001375957437049947</v>
+        <v>3.10525023880853e-05</v>
       </c>
       <c r="T18" s="7" t="n">
         <v>1554</v>
@@ -1836,7 +1836,7 @@
         <v>9</v>
       </c>
       <c r="W18" s="6" t="n">
-        <v>1.37725238149891e-05</v>
+        <v>1.396158392618356e-05</v>
       </c>
       <c r="X18" s="7" t="n">
         <v>837</v>
@@ -1848,7 +1848,7 @@
         <v>72</v>
       </c>
       <c r="BG18" s="6" t="n">
-        <v>2.796119762469626e-05</v>
+        <v>2.396039346959476e-05</v>
       </c>
       <c r="BH18" s="10" t="n">
         <v>5499</v>
@@ -1910,7 +1910,7 @@
         <v>769</v>
       </c>
       <c r="K20" s="6" t="n">
-        <v>0.0007674482196997671</v>
+        <v>0.0007737539442333698</v>
       </c>
       <c r="L20" s="7" t="n">
         <v>159805.2</v>
@@ -1922,7 +1922,7 @@
         <v>769</v>
       </c>
       <c r="BG20" s="6" t="n">
-        <v>0.0002986411246304364</v>
+        <v>0.0002559103135849774</v>
       </c>
       <c r="BH20" s="10" t="n">
         <v>159805.2</v>
@@ -2046,7 +2046,7 @@
         <v>252</v>
       </c>
       <c r="W24" s="6" t="n">
-        <v>0.0003856306668196947</v>
+        <v>0.0003909243499331395</v>
       </c>
       <c r="X24" s="7" t="n">
         <v>344079.51</v>
@@ -2058,7 +2058,7 @@
         <v>252</v>
       </c>
       <c r="BG24" s="6" t="n">
-        <v>9.786419168643692e-05</v>
+        <v>8.386137714358165e-05</v>
       </c>
       <c r="BH24" s="10" t="n">
         <v>844079.51</v>
@@ -2070,29 +2070,29 @@
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>CLIENTE: PROVINCIA ART (nuevo 2026)</t>
+          <t>CLIENTE: AVANTER</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>5310</t>
+          <t>5004</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Provincia ART</t>
+          <t>Programa TEVAcuidar (TEVA)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>PROVINCIA ART</t>
+          <t>TEVA</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
@@ -2100,15 +2100,19 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr"/>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>SI - ETICOS</t>
+        </is>
+      </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>0,35% sobre monto vendido</t>
+          <t>Facturado vía Avanter - valor unitario por TRX</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Mensual</t>
+          <t>Trimestral por IPC Indec</t>
         </is>
       </c>
       <c r="I26" s="4" t="inlineStr">
@@ -2117,80 +2121,192 @@
         </is>
       </c>
       <c r="J26" s="5" t="n">
-        <v>8166</v>
+        <v>147</v>
       </c>
       <c r="K26" s="6" t="n">
-        <v>0.008149521667188945</v>
+        <v>0.0001479087513684075</v>
       </c>
       <c r="L26" s="7" t="n">
-        <v>1073509.3</v>
+        <v>10878</v>
       </c>
       <c r="M26" s="8" t="n">
-        <v>131.4608498652951</v>
+        <v>74</v>
+      </c>
+      <c r="N26" s="5" t="n">
+        <v>135</v>
+      </c>
+      <c r="O26" s="6" t="n">
+        <v>0.0001955946294061312</v>
+      </c>
+      <c r="P26" s="7" t="n">
+        <v>9990</v>
+      </c>
+      <c r="Q26" s="8" t="n">
+        <v>74</v>
       </c>
       <c r="R26" s="5" t="n">
-        <v>8692</v>
+        <v>172</v>
       </c>
       <c r="S26" s="6" t="n">
-        <v>0.05695153353732448</v>
+        <v>0.0002543347814643177</v>
       </c>
       <c r="T26" s="7" t="n">
-        <v>1293685.98</v>
+        <v>12728</v>
       </c>
       <c r="U26" s="8" t="n">
-        <v>148.8363989875748</v>
+        <v>74</v>
       </c>
       <c r="V26" s="5" t="n">
-        <v>8849</v>
+        <v>150</v>
       </c>
       <c r="W26" s="6" t="n">
-        <v>0.01354145147098206</v>
+        <v>0.0002326930654363926</v>
       </c>
       <c r="X26" s="7" t="n">
-        <v>1471007.21</v>
+        <v>13950</v>
       </c>
       <c r="Y26" s="8" t="n">
-        <v>166.2342874901119</v>
+        <v>93</v>
       </c>
       <c r="BF26" s="9" t="n">
-        <v>25707</v>
+        <v>604</v>
       </c>
       <c r="BG26" s="6" t="n">
-        <v>0.009983312601917595</v>
+        <v>0.0002010010785504894</v>
       </c>
       <c r="BH26" s="10" t="n">
-        <v>3838202.49</v>
+        <v>47546</v>
       </c>
       <c r="BI26" s="8" t="n">
-        <v>149.3057334578131</v>
+        <v>78.71854304635761</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
-          <t>CLIENTE: SERDATA (nuevo 2026)</t>
-        </is>
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>5010</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Bonos Loreal</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>LOREAL</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>SI - DINAMICAS - BONOS</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Facturado vía Avanter - valor unitario por TRX</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Trimestral por IPC Indec</t>
+        </is>
+      </c>
+      <c r="I27" s="4" t="inlineStr">
+        <is>
+          <t>PRODUCTIVO</t>
+        </is>
+      </c>
+      <c r="J27" s="5" t="n">
+        <v>91364</v>
+      </c>
+      <c r="K27" s="6" t="n">
+        <v>0.0919288106124026</v>
+      </c>
+      <c r="L27" s="7" t="n">
+        <v>6760936</v>
+      </c>
+      <c r="M27" s="8" t="n">
+        <v>74</v>
+      </c>
+      <c r="N27" s="5" t="n">
+        <v>74721</v>
+      </c>
+      <c r="O27" s="6" t="n">
+        <v>0.1082594541026336</v>
+      </c>
+      <c r="P27" s="7" t="n">
+        <v>5529354</v>
+      </c>
+      <c r="Q27" s="8" t="n">
+        <v>74</v>
+      </c>
+      <c r="R27" s="5" t="n">
+        <v>75325</v>
+      </c>
+      <c r="S27" s="6" t="n">
+        <v>0.1113823686848822</v>
+      </c>
+      <c r="T27" s="7" t="n">
+        <v>5574050</v>
+      </c>
+      <c r="U27" s="8" t="n">
+        <v>74</v>
+      </c>
+      <c r="V27" s="5" t="n">
+        <v>67206</v>
+      </c>
+      <c r="W27" s="6" t="n">
+        <v>0.1042558010381213</v>
+      </c>
+      <c r="X27" s="7" t="n">
+        <v>6250158</v>
+      </c>
+      <c r="Y27" s="8" t="n">
+        <v>93</v>
+      </c>
+      <c r="BF27" s="9" t="n">
+        <v>308616</v>
+      </c>
+      <c r="BG27" s="6" t="n">
+        <v>0.1027022332085063</v>
+      </c>
+      <c r="BH27" s="10" t="n">
+        <v>24114498</v>
+      </c>
+      <c r="BI27" s="8" t="n">
+        <v>78.13754957617233</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>5320</t>
+          <t>5011</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Serdata (Bonos)</t>
+          <t>Programa Beneficiarte (Ferring)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>SERDATA</t>
+          <t>FERRING</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
@@ -2198,15 +2314,19 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr"/>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>SI - ETICOS</t>
+        </is>
+      </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Valor unitario por bono procesado</t>
+          <t>Facturado vía Avanter - valor unitario por TRX</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Mensual</t>
+          <t>Trimestral por IPC Indec</t>
         </is>
       </c>
       <c r="I28" s="4" t="inlineStr">
@@ -2214,52 +2334,188 @@
           <t>PRODUCTIVO</t>
         </is>
       </c>
+      <c r="J28" s="5" t="n">
+        <v>453</v>
+      </c>
+      <c r="K28" s="6" t="n">
+        <v>0.0004558004378903986</v>
+      </c>
+      <c r="L28" s="7" t="n">
+        <v>33522</v>
+      </c>
+      <c r="M28" s="8" t="n">
+        <v>74</v>
+      </c>
       <c r="N28" s="5" t="n">
-        <v>76676</v>
+        <v>394</v>
       </c>
       <c r="O28" s="6" t="n">
-        <v>0.09998448255852618</v>
+        <v>0.0005708465480445608</v>
       </c>
       <c r="P28" s="7" t="n">
-        <v>4544586.52</v>
+        <v>29156</v>
       </c>
       <c r="Q28" s="8" t="n">
-        <v>59.27</v>
+        <v>74</v>
+      </c>
+      <c r="R28" s="5" t="n">
+        <v>518</v>
+      </c>
+      <c r="S28" s="6" t="n">
+        <v>0.0007659617255727708</v>
+      </c>
+      <c r="T28" s="7" t="n">
+        <v>38332</v>
+      </c>
+      <c r="U28" s="8" t="n">
+        <v>74</v>
+      </c>
+      <c r="V28" s="5" t="n">
+        <v>484</v>
+      </c>
+      <c r="W28" s="6" t="n">
+        <v>0.0007508229578080934</v>
+      </c>
+      <c r="X28" s="7" t="n">
+        <v>45012</v>
+      </c>
+      <c r="Y28" s="8" t="n">
+        <v>93</v>
       </c>
       <c r="BF28" s="9" t="n">
-        <v>76676</v>
+        <v>1849</v>
       </c>
       <c r="BG28" s="6" t="n">
-        <v>0.02977712207043348</v>
+        <v>0.0006153162156288987</v>
       </c>
       <c r="BH28" s="10" t="n">
-        <v>4544586.52</v>
+        <v>146022</v>
       </c>
       <c r="BI28" s="8" t="n">
-        <v>59.27</v>
+        <v>78.97349918875068</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="3" t="inlineStr">
-        <is>
-          <t>CLIENTE: AVANTER</t>
-        </is>
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>5014</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Programa Rossmore</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>ROSSMORE</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>SI - ETICOS</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Facturado vía Avanter - valor unitario por TRX</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Trimestral por IPC Indec</t>
+        </is>
+      </c>
+      <c r="I29" s="4" t="inlineStr">
+        <is>
+          <t>PRODUCTIVO</t>
+        </is>
+      </c>
+      <c r="J29" s="5" t="n">
+        <v>1549</v>
+      </c>
+      <c r="K29" s="6" t="n">
+        <v>0.001558575890269818</v>
+      </c>
+      <c r="L29" s="7" t="n">
+        <v>114626</v>
+      </c>
+      <c r="M29" s="8" t="n">
+        <v>74</v>
+      </c>
+      <c r="N29" s="5" t="n">
+        <v>1437</v>
+      </c>
+      <c r="O29" s="6" t="n">
+        <v>0.002081996166345264</v>
+      </c>
+      <c r="P29" s="7" t="n">
+        <v>106338</v>
+      </c>
+      <c r="Q29" s="8" t="n">
+        <v>74</v>
+      </c>
+      <c r="R29" s="5" t="n">
+        <v>1708</v>
+      </c>
+      <c r="S29" s="6" t="n">
+        <v>0.002525603527564271</v>
+      </c>
+      <c r="T29" s="7" t="n">
+        <v>126392</v>
+      </c>
+      <c r="U29" s="8" t="n">
+        <v>74</v>
+      </c>
+      <c r="V29" s="5" t="n">
+        <v>1683</v>
+      </c>
+      <c r="W29" s="6" t="n">
+        <v>0.002610816194196325</v>
+      </c>
+      <c r="X29" s="7" t="n">
+        <v>156519</v>
+      </c>
+      <c r="Y29" s="8" t="n">
+        <v>93</v>
+      </c>
+      <c r="BF29" s="9" t="n">
+        <v>6377</v>
+      </c>
+      <c r="BG29" s="6" t="n">
+        <v>0.002122158738272303</v>
+      </c>
+      <c r="BH29" s="10" t="n">
+        <v>503875</v>
+      </c>
+      <c r="BI29" s="8" t="n">
+        <v>79.01442684647954</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>5004</t>
+          <t>5020</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Programa TEVAcuidar (TEVA)</t>
+          <t>Bonos Eucerin</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>TEVA</t>
+          <t>BEIERSDORF</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
@@ -2274,7 +2530,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>SI - ETICOS</t>
+          <t>SI - DINAMICAS - BONOS</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -2293,68 +2549,80 @@
         </is>
       </c>
       <c r="J30" s="5" t="n">
-        <v>147</v>
+        <v>42157</v>
       </c>
       <c r="K30" s="6" t="n">
-        <v>0.0001467033657943638</v>
+        <v>0.04241761381930582</v>
       </c>
       <c r="L30" s="7" t="n">
-        <v>10878</v>
+        <v>3119618</v>
       </c>
       <c r="M30" s="8" t="n">
         <v>74</v>
       </c>
       <c r="N30" s="5" t="n">
-        <v>135</v>
+        <v>30505</v>
       </c>
       <c r="O30" s="6" t="n">
-        <v>0.0001760382015937325</v>
+        <v>0.0441971420002521</v>
       </c>
       <c r="P30" s="7" t="n">
-        <v>9990</v>
+        <v>2257370</v>
       </c>
       <c r="Q30" s="8" t="n">
         <v>74</v>
       </c>
+      <c r="R30" s="5" t="n">
+        <v>34604</v>
+      </c>
+      <c r="S30" s="6" t="n">
+        <v>0.05116860917320494</v>
+      </c>
+      <c r="T30" s="7" t="n">
+        <v>2560696</v>
+      </c>
+      <c r="U30" s="8" t="n">
+        <v>74</v>
+      </c>
       <c r="V30" s="5" t="n">
-        <v>150</v>
+        <v>29074</v>
       </c>
       <c r="W30" s="6" t="n">
-        <v>0.0002295420635831516</v>
+        <v>0.04510212122998452</v>
       </c>
       <c r="X30" s="7" t="n">
-        <v>13950</v>
+        <v>2703882</v>
       </c>
       <c r="Y30" s="8" t="n">
         <v>93</v>
       </c>
       <c r="BF30" s="9" t="n">
-        <v>432</v>
+        <v>136340</v>
       </c>
       <c r="BG30" s="6" t="n">
-        <v>0.0001677671857481776</v>
+        <v>0.04537166730061874</v>
       </c>
       <c r="BH30" s="10" t="n">
-        <v>34818</v>
+        <v>10641566</v>
       </c>
       <c r="BI30" s="8" t="n">
-        <v>80.59722222222223</v>
+        <v>78.05167962446824</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>5010</t>
+          <t>5022</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Bonos Loreal</t>
+          <t>Ofertas Casasco</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>LOREAL</t>
+          <t>CASASCO</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
@@ -2388,68 +2656,80 @@
         </is>
       </c>
       <c r="J31" s="5" t="n">
-        <v>91364</v>
+        <v>34587</v>
       </c>
       <c r="K31" s="6" t="n">
-        <v>0.09117963477847792</v>
+        <v>0.03480081621482388</v>
       </c>
       <c r="L31" s="7" t="n">
-        <v>6760936</v>
+        <v>2559438</v>
       </c>
       <c r="M31" s="8" t="n">
         <v>74</v>
       </c>
       <c r="N31" s="5" t="n">
-        <v>74721</v>
+        <v>28811</v>
       </c>
       <c r="O31" s="6" t="n">
-        <v>0.09743518860211324</v>
+        <v>0.04174279161348183</v>
       </c>
       <c r="P31" s="7" t="n">
-        <v>5529354</v>
+        <v>2132014</v>
       </c>
       <c r="Q31" s="8" t="n">
         <v>74</v>
       </c>
+      <c r="R31" s="5" t="n">
+        <v>28256</v>
+      </c>
+      <c r="S31" s="6" t="n">
+        <v>0.04178188130846373</v>
+      </c>
+      <c r="T31" s="7" t="n">
+        <v>2090944</v>
+      </c>
+      <c r="U31" s="8" t="n">
+        <v>74</v>
+      </c>
       <c r="V31" s="5" t="n">
-        <v>67206</v>
+        <v>25273</v>
       </c>
       <c r="W31" s="6" t="n">
-        <v>0.1028440261677953</v>
+        <v>0.03920567895182633</v>
       </c>
       <c r="X31" s="7" t="n">
-        <v>6250158</v>
+        <v>2350389</v>
       </c>
       <c r="Y31" s="8" t="n">
         <v>93</v>
       </c>
       <c r="BF31" s="9" t="n">
-        <v>233291</v>
+        <v>116927</v>
       </c>
       <c r="BG31" s="6" t="n">
-        <v>0.09059855215365299</v>
+        <v>0.03891134621137925</v>
       </c>
       <c r="BH31" s="10" t="n">
-        <v>18540448</v>
+        <v>9132785</v>
       </c>
       <c r="BI31" s="8" t="n">
-        <v>79.47348161737915</v>
+        <v>78.10672470857885</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>5011</t>
+          <t>5023</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Programa Beneficiarte (Ferring)</t>
+          <t>Programa Farmaspen (Aspen)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>FERRING</t>
+          <t>ASPEN</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
@@ -2483,68 +2763,80 @@
         </is>
       </c>
       <c r="J32" s="5" t="n">
-        <v>453</v>
+        <v>1991</v>
       </c>
       <c r="K32" s="6" t="n">
-        <v>0.0004520858823458966</v>
+        <v>0.002003308326357138</v>
       </c>
       <c r="L32" s="7" t="n">
-        <v>33522</v>
+        <v>147334</v>
       </c>
       <c r="M32" s="8" t="n">
         <v>74</v>
       </c>
       <c r="N32" s="5" t="n">
-        <v>394</v>
+        <v>1778</v>
       </c>
       <c r="O32" s="6" t="n">
-        <v>0.0005137707513180045</v>
+        <v>0.002576053711734084</v>
       </c>
       <c r="P32" s="7" t="n">
-        <v>29156</v>
+        <v>131572</v>
       </c>
       <c r="Q32" s="8" t="n">
         <v>74</v>
       </c>
+      <c r="R32" s="5" t="n">
+        <v>2097</v>
+      </c>
+      <c r="S32" s="6" t="n">
+        <v>0.003100814167038804</v>
+      </c>
+      <c r="T32" s="7" t="n">
+        <v>155178</v>
+      </c>
+      <c r="U32" s="8" t="n">
+        <v>74</v>
+      </c>
       <c r="V32" s="5" t="n">
-        <v>484</v>
+        <v>2285</v>
       </c>
       <c r="W32" s="6" t="n">
-        <v>0.0007406557251616358</v>
+        <v>0.003544691030147714</v>
       </c>
       <c r="X32" s="7" t="n">
-        <v>45012</v>
+        <v>212505</v>
       </c>
       <c r="Y32" s="8" t="n">
         <v>93</v>
       </c>
       <c r="BF32" s="9" t="n">
-        <v>1331</v>
+        <v>8151</v>
       </c>
       <c r="BG32" s="6" t="n">
-        <v>0.0005168938060898712</v>
+        <v>0.002712516210703707</v>
       </c>
       <c r="BH32" s="10" t="n">
-        <v>107690</v>
+        <v>646589</v>
       </c>
       <c r="BI32" s="8" t="n">
-        <v>80.90909090909091</v>
+        <v>79.32634032634033</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>5014</t>
+          <t>5024</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Programa Rossmore</t>
+          <t>Nutricia Siempre Juntos (Bagó)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>ROSSMORE</t>
+          <t>BAGO</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
@@ -2578,68 +2870,80 @@
         </is>
       </c>
       <c r="J33" s="5" t="n">
-        <v>1549</v>
+        <v>387</v>
       </c>
       <c r="K33" s="6" t="n">
-        <v>0.001545874242282106</v>
+        <v>0.0003893924270719299</v>
       </c>
       <c r="L33" s="7" t="n">
-        <v>114626</v>
+        <v>28638</v>
       </c>
       <c r="M33" s="8" t="n">
         <v>74</v>
       </c>
       <c r="N33" s="5" t="n">
-        <v>1437</v>
+        <v>329</v>
       </c>
       <c r="O33" s="6" t="n">
-        <v>0.001873828856964397</v>
+        <v>0.0004766713561082754</v>
       </c>
       <c r="P33" s="7" t="n">
-        <v>106338</v>
+        <v>24346</v>
       </c>
       <c r="Q33" s="8" t="n">
         <v>74</v>
       </c>
+      <c r="R33" s="5" t="n">
+        <v>383</v>
+      </c>
+      <c r="S33" s="6" t="n">
+        <v>0.0005663384959350796</v>
+      </c>
+      <c r="T33" s="7" t="n">
+        <v>28342</v>
+      </c>
+      <c r="U33" s="8" t="n">
+        <v>74</v>
+      </c>
       <c r="V33" s="5" t="n">
-        <v>1683</v>
+        <v>421</v>
       </c>
       <c r="W33" s="6" t="n">
-        <v>0.002575461953402961</v>
+        <v>0.0006530918703248085</v>
       </c>
       <c r="X33" s="7" t="n">
-        <v>156519</v>
+        <v>39153</v>
       </c>
       <c r="Y33" s="8" t="n">
         <v>93</v>
       </c>
       <c r="BF33" s="9" t="n">
-        <v>4669</v>
+        <v>1520</v>
       </c>
       <c r="BG33" s="6" t="n">
-        <v>0.001813205995968151</v>
+        <v>0.0005058305288025561</v>
       </c>
       <c r="BH33" s="10" t="n">
-        <v>377483</v>
+        <v>120479</v>
       </c>
       <c r="BI33" s="8" t="n">
-        <v>80.8487898907689</v>
+        <v>79.2625</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>5020</t>
+          <t>5027</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Bonos Eucerin</t>
+          <t>Programa Vari Te Acerca (Varifarma)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>BEIERSDORF</t>
+          <t>VARIFARMA</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
@@ -2654,7 +2958,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>SI - DINAMICAS - BONOS</t>
+          <t>SI - ETICOS</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2673,68 +2977,80 @@
         </is>
       </c>
       <c r="J34" s="5" t="n">
-        <v>42157</v>
+        <v>7</v>
       </c>
       <c r="K34" s="6" t="n">
-        <v>0.04207193055641493</v>
+        <v>7.043273874686071e-06</v>
       </c>
       <c r="L34" s="7" t="n">
-        <v>3119618</v>
+        <v>518</v>
       </c>
       <c r="M34" s="8" t="n">
         <v>74</v>
       </c>
       <c r="N34" s="5" t="n">
-        <v>30505</v>
+        <v>6</v>
       </c>
       <c r="O34" s="6" t="n">
-        <v>0.03977811362679119</v>
+        <v>8.6930946402725e-06</v>
       </c>
       <c r="P34" s="7" t="n">
-        <v>2257370</v>
+        <v>444</v>
       </c>
       <c r="Q34" s="8" t="n">
         <v>74</v>
       </c>
+      <c r="R34" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="S34" s="6" t="n">
+        <v>1.182952471927059e-05</v>
+      </c>
+      <c r="T34" s="7" t="n">
+        <v>592</v>
+      </c>
+      <c r="U34" s="8" t="n">
+        <v>74</v>
+      </c>
       <c r="V34" s="5" t="n">
-        <v>29074</v>
+        <v>8</v>
       </c>
       <c r="W34" s="6" t="n">
-        <v>0.04449137304411033</v>
+        <v>1.241029682327427e-05</v>
       </c>
       <c r="X34" s="7" t="n">
-        <v>2703882</v>
+        <v>744</v>
       </c>
       <c r="Y34" s="8" t="n">
         <v>93</v>
       </c>
       <c r="BF34" s="9" t="n">
-        <v>101736</v>
+        <v>29</v>
       </c>
       <c r="BG34" s="6" t="n">
-        <v>0.03950917224369582</v>
+        <v>9.650714036364556e-06</v>
       </c>
       <c r="BH34" s="10" t="n">
-        <v>8080870</v>
+        <v>2298</v>
       </c>
       <c r="BI34" s="8" t="n">
-        <v>79.42979869466069</v>
+        <v>79.24137931034483</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>5022</t>
+          <t>5050</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Ofertas Casasco</t>
+          <t>Bonos Andrómaco</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>CASASCO</t>
+          <t>ANDROMACO</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
@@ -2768,68 +3084,80 @@
         </is>
       </c>
       <c r="J35" s="5" t="n">
-        <v>34587</v>
+        <v>554837</v>
       </c>
       <c r="K35" s="6" t="n">
-        <v>0.03451720620904531</v>
+        <v>0.5582669924013137</v>
       </c>
       <c r="L35" s="7" t="n">
-        <v>2559438</v>
+        <v>41057938</v>
       </c>
       <c r="M35" s="8" t="n">
         <v>74</v>
       </c>
       <c r="N35" s="5" t="n">
-        <v>28811</v>
+        <v>336212</v>
       </c>
       <c r="O35" s="6" t="n">
-        <v>0.03756916019345946</v>
+        <v>0.4871204558658829</v>
       </c>
       <c r="P35" s="7" t="n">
-        <v>2132014</v>
+        <v>24879688</v>
       </c>
       <c r="Q35" s="8" t="n">
         <v>74</v>
       </c>
+      <c r="R35" s="5" t="n">
+        <v>274190</v>
+      </c>
+      <c r="S35" s="6" t="n">
+        <v>0.4054421728471004</v>
+      </c>
+      <c r="T35" s="7" t="n">
+        <v>20290060</v>
+      </c>
+      <c r="U35" s="8" t="n">
+        <v>74</v>
+      </c>
       <c r="V35" s="5" t="n">
-        <v>25273</v>
+        <v>260641</v>
       </c>
       <c r="W35" s="6" t="n">
-        <v>0.03867477715291327</v>
+        <v>0.4043290217893786</v>
       </c>
       <c r="X35" s="7" t="n">
-        <v>2350389</v>
+        <v>24239613</v>
       </c>
       <c r="Y35" s="8" t="n">
         <v>93</v>
       </c>
       <c r="BF35" s="9" t="n">
-        <v>88671</v>
+        <v>1425880</v>
       </c>
       <c r="BG35" s="6" t="n">
-        <v>0.03443537992471447</v>
+        <v>0.4745089700059136</v>
       </c>
       <c r="BH35" s="10" t="n">
-        <v>7041841</v>
+        <v>110467299</v>
       </c>
       <c r="BI35" s="8" t="n">
-        <v>79.41537819580246</v>
+        <v>77.47306856116924</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>5023</t>
+          <t>5060</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Programa Farmaspen (Aspen)</t>
+          <t>Bonos Isdin</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ASPEN</t>
+          <t>ISDIN</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
@@ -2844,7 +3172,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>SI - ETICOS</t>
+          <t>SI - DINAMICAS - BONOS</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2863,68 +3191,80 @@
         </is>
       </c>
       <c r="J36" s="5" t="n">
-        <v>1991</v>
+        <v>40175</v>
       </c>
       <c r="K36" s="6" t="n">
-        <v>0.001986982321745431</v>
+        <v>0.04042336113078756</v>
       </c>
       <c r="L36" s="7" t="n">
-        <v>147334</v>
+        <v>2972950</v>
       </c>
       <c r="M36" s="8" t="n">
         <v>74</v>
       </c>
       <c r="N36" s="5" t="n">
-        <v>1778</v>
+        <v>25065</v>
       </c>
       <c r="O36" s="6" t="n">
-        <v>0.002318488314323381</v>
+        <v>0.03631540285973837</v>
       </c>
       <c r="P36" s="7" t="n">
-        <v>131572</v>
+        <v>1854810</v>
       </c>
       <c r="Q36" s="8" t="n">
         <v>74</v>
       </c>
+      <c r="R36" s="5" t="n">
+        <v>21680</v>
+      </c>
+      <c r="S36" s="6" t="n">
+        <v>0.0320580119892233</v>
+      </c>
+      <c r="T36" s="7" t="n">
+        <v>1604320</v>
+      </c>
+      <c r="U36" s="8" t="n">
+        <v>74</v>
+      </c>
       <c r="V36" s="5" t="n">
-        <v>2285</v>
+        <v>18937</v>
       </c>
       <c r="W36" s="6" t="n">
-        <v>0.003496690768583343</v>
+        <v>0.02937672386779311</v>
       </c>
       <c r="X36" s="7" t="n">
-        <v>212505</v>
+        <v>1761141</v>
       </c>
       <c r="Y36" s="8" t="n">
         <v>93</v>
       </c>
       <c r="BF36" s="9" t="n">
-        <v>6054</v>
+        <v>105857</v>
       </c>
       <c r="BG36" s="6" t="n">
-        <v>0.002351070700276544</v>
+        <v>0.03522743571542906</v>
       </c>
       <c r="BH36" s="10" t="n">
-        <v>491411</v>
+        <v>8193221</v>
       </c>
       <c r="BI36" s="8" t="n">
-        <v>81.17129170796167</v>
+        <v>77.39895330493023</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>5024</t>
+          <t>5090</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Nutricia Siempre Juntos (Bagó)</t>
+          <t>Bonos Galderma</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>BAGO</t>
+          <t>GALDERMA</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
@@ -2939,7 +3279,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>SI - ETICOS</t>
+          <t>SI - DINAMICAS - BONOS</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2958,68 +3298,80 @@
         </is>
       </c>
       <c r="J37" s="5" t="n">
-        <v>387</v>
+        <v>10966</v>
       </c>
       <c r="K37" s="6" t="n">
-        <v>0.000386219065050468</v>
+        <v>0.01103379161568678</v>
       </c>
       <c r="L37" s="7" t="n">
-        <v>28638</v>
+        <v>811484</v>
       </c>
       <c r="M37" s="8" t="n">
         <v>74</v>
       </c>
       <c r="N37" s="5" t="n">
-        <v>329</v>
+        <v>7941</v>
       </c>
       <c r="O37" s="6" t="n">
-        <v>0.0004290116172173185</v>
+        <v>0.01150531075640065</v>
       </c>
       <c r="P37" s="7" t="n">
-        <v>24346</v>
+        <v>587634</v>
       </c>
       <c r="Q37" s="8" t="n">
         <v>74</v>
       </c>
+      <c r="R37" s="5" t="n">
+        <v>10088</v>
+      </c>
+      <c r="S37" s="6" t="n">
+        <v>0.01491703067100022</v>
+      </c>
+      <c r="T37" s="7" t="n">
+        <v>746512</v>
+      </c>
+      <c r="U37" s="8" t="n">
+        <v>74</v>
+      </c>
       <c r="V37" s="5" t="n">
-        <v>421</v>
+        <v>9934</v>
       </c>
       <c r="W37" s="6" t="n">
-        <v>0.0006442480584567122</v>
+        <v>0.01541048608030083</v>
       </c>
       <c r="X37" s="7" t="n">
-        <v>39153</v>
+        <v>923862</v>
       </c>
       <c r="Y37" s="8" t="n">
         <v>93</v>
       </c>
       <c r="BF37" s="9" t="n">
-        <v>1137</v>
+        <v>38929</v>
       </c>
       <c r="BG37" s="6" t="n">
-        <v>0.0004415539124899952</v>
+        <v>0.0129549188524702</v>
       </c>
       <c r="BH37" s="10" t="n">
-        <v>92137</v>
+        <v>3069492</v>
       </c>
       <c r="BI37" s="8" t="n">
-        <v>81.03518029903255</v>
+        <v>78.84846772329112</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>5027</t>
+          <t>5100</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Programa Vari Te Acerca (Varifarma)</t>
+          <t>Bonos Bernabo</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>VARIFARMA</t>
+          <t>BERNABO</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
@@ -3034,7 +3386,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>SI - ETICOS</t>
+          <t>SI - DINAMICAS - BONOS</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -3053,68 +3405,80 @@
         </is>
       </c>
       <c r="J38" s="5" t="n">
-        <v>7</v>
+        <v>4458</v>
       </c>
       <c r="K38" s="6" t="n">
-        <v>6.985874561636371e-06</v>
+        <v>0.00448555927619293</v>
       </c>
       <c r="L38" s="7" t="n">
-        <v>518</v>
+        <v>329892</v>
       </c>
       <c r="M38" s="8" t="n">
         <v>74</v>
       </c>
       <c r="N38" s="5" t="n">
-        <v>6</v>
+        <v>4207</v>
       </c>
       <c r="O38" s="6" t="n">
-        <v>7.823920070832557e-06</v>
+        <v>0.006095308191937735</v>
       </c>
       <c r="P38" s="7" t="n">
-        <v>444</v>
+        <v>311318</v>
       </c>
       <c r="Q38" s="8" t="n">
         <v>74</v>
       </c>
+      <c r="R38" s="5" t="n">
+        <v>4609</v>
+      </c>
+      <c r="S38" s="6" t="n">
+        <v>0.006815284928889769</v>
+      </c>
+      <c r="T38" s="7" t="n">
+        <v>341066</v>
+      </c>
+      <c r="U38" s="8" t="n">
+        <v>74</v>
+      </c>
       <c r="V38" s="5" t="n">
-        <v>8</v>
+        <v>4464</v>
       </c>
       <c r="W38" s="6" t="n">
-        <v>1.224224339110142e-05</v>
+        <v>0.006924945627387043</v>
       </c>
       <c r="X38" s="7" t="n">
-        <v>744</v>
+        <v>415152</v>
       </c>
       <c r="Y38" s="8" t="n">
         <v>93</v>
       </c>
       <c r="BF38" s="9" t="n">
-        <v>21</v>
+        <v>17738</v>
       </c>
       <c r="BG38" s="6" t="n">
-        <v>8.155349307203077e-06</v>
+        <v>0.005902909157828776</v>
       </c>
       <c r="BH38" s="10" t="n">
-        <v>1706</v>
+        <v>1397428</v>
       </c>
       <c r="BI38" s="8" t="n">
-        <v>81.23809523809524</v>
+        <v>78.78159882737626</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>5050</t>
+          <t>5110</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Bonos Andrómaco</t>
+          <t>Bonos Eurolab</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>ANDROMACO</t>
+          <t>EUROLAB</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
@@ -3148,68 +3512,80 @@
         </is>
       </c>
       <c r="J39" s="5" t="n">
-        <v>554837</v>
+        <v>26534</v>
       </c>
       <c r="K39" s="6" t="n">
-        <v>0.5537173834506628</v>
+        <v>0.0266980327129886</v>
       </c>
       <c r="L39" s="7" t="n">
-        <v>41057938</v>
+        <v>1963516</v>
       </c>
       <c r="M39" s="8" t="n">
         <v>74</v>
       </c>
       <c r="N39" s="5" t="n">
-        <v>336212</v>
+        <v>24819</v>
       </c>
       <c r="O39" s="6" t="n">
-        <v>0.4384159691424592</v>
+        <v>0.03595898597948719</v>
       </c>
       <c r="P39" s="7" t="n">
-        <v>24879688</v>
+        <v>1836606</v>
       </c>
       <c r="Q39" s="8" t="n">
         <v>74</v>
       </c>
+      <c r="R39" s="5" t="n">
+        <v>30701</v>
+      </c>
+      <c r="S39" s="6" t="n">
+        <v>0.0453972798007908</v>
+      </c>
+      <c r="T39" s="7" t="n">
+        <v>2271874</v>
+      </c>
+      <c r="U39" s="8" t="n">
+        <v>74</v>
+      </c>
       <c r="V39" s="5" t="n">
-        <v>260641</v>
+        <v>31434</v>
       </c>
       <c r="W39" s="6" t="n">
-        <v>0.3988538199625081</v>
+        <v>0.04876315879285043</v>
       </c>
       <c r="X39" s="7" t="n">
-        <v>24239613</v>
+        <v>2923362</v>
       </c>
       <c r="Y39" s="8" t="n">
         <v>93</v>
       </c>
       <c r="BF39" s="9" t="n">
-        <v>1151690</v>
+        <v>113488</v>
       </c>
       <c r="BG39" s="6" t="n">
-        <v>0.4472587735053672</v>
+        <v>0.03776690463996348</v>
       </c>
       <c r="BH39" s="10" t="n">
-        <v>90177239</v>
+        <v>8995358</v>
       </c>
       <c r="BI39" s="8" t="n">
-        <v>78.29992359054954</v>
+        <v>79.26263569716622</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>5060</t>
+          <t>5120</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Bonos Isdin</t>
+          <t>Eximia Cepage (Ceoderma) - vía Avanter</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>ISDIN</t>
+          <t>CEODERMA</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
@@ -3224,7 +3600,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>SI - DINAMICAS - BONOS</t>
+          <t>SI - ETICOS</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -3243,68 +3619,44 @@
         </is>
       </c>
       <c r="J40" s="5" t="n">
-        <v>40175</v>
+        <v>355</v>
       </c>
       <c r="K40" s="6" t="n">
-        <v>0.04009393007339161</v>
+        <v>0.0003571946036447936</v>
       </c>
       <c r="L40" s="7" t="n">
-        <v>2972950</v>
+        <v>26270</v>
       </c>
       <c r="M40" s="8" t="n">
         <v>74</v>
       </c>
-      <c r="N40" s="5" t="n">
-        <v>25065</v>
-      </c>
-      <c r="O40" s="6" t="n">
-        <v>0.032684426095903</v>
-      </c>
-      <c r="P40" s="7" t="n">
-        <v>1854810</v>
-      </c>
-      <c r="Q40" s="8" t="n">
-        <v>74</v>
-      </c>
-      <c r="V40" s="5" t="n">
-        <v>18937</v>
-      </c>
-      <c r="W40" s="6" t="n">
-        <v>0.02897892038716095</v>
-      </c>
-      <c r="X40" s="7" t="n">
-        <v>1761141</v>
-      </c>
-      <c r="Y40" s="8" t="n">
-        <v>93</v>
-      </c>
       <c r="BF40" s="9" t="n">
-        <v>84177</v>
+        <v>355</v>
       </c>
       <c r="BG40" s="6" t="n">
-        <v>0.03269013517297302</v>
+        <v>0.0001181380511348075</v>
       </c>
       <c r="BH40" s="10" t="n">
-        <v>6588901</v>
+        <v>26270</v>
       </c>
       <c r="BI40" s="8" t="n">
-        <v>78.27436235551279</v>
+        <v>74</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>5090</t>
+          <t>5130</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Bonos Galderma</t>
+          <t>Bonos Cassara</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>GALDERMA</t>
+          <t>CASSARA</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
@@ -3338,68 +3690,80 @@
         </is>
       </c>
       <c r="J41" s="5" t="n">
-        <v>10966</v>
+        <v>8603</v>
       </c>
       <c r="K41" s="6" t="n">
-        <v>0.01094387149184349</v>
+        <v>0.008656183591989181</v>
       </c>
       <c r="L41" s="7" t="n">
-        <v>811484</v>
+        <v>636622</v>
       </c>
       <c r="M41" s="8" t="n">
         <v>74</v>
       </c>
       <c r="N41" s="5" t="n">
-        <v>7941</v>
+        <v>7894</v>
       </c>
       <c r="O41" s="6" t="n">
-        <v>0.01035495821374689</v>
+        <v>0.01143721484838518</v>
       </c>
       <c r="P41" s="7" t="n">
-        <v>587634</v>
+        <v>584156</v>
       </c>
       <c r="Q41" s="8" t="n">
         <v>74</v>
       </c>
+      <c r="R41" s="5" t="n">
+        <v>9727</v>
+      </c>
+      <c r="S41" s="6" t="n">
+        <v>0.01438322336804313</v>
+      </c>
+      <c r="T41" s="7" t="n">
+        <v>719798</v>
+      </c>
+      <c r="U41" s="8" t="n">
+        <v>74</v>
+      </c>
       <c r="V41" s="5" t="n">
-        <v>9934</v>
+        <v>9823</v>
       </c>
       <c r="W41" s="6" t="n">
-        <v>0.01520180573090019</v>
+        <v>0.0152382932118779</v>
       </c>
       <c r="X41" s="7" t="n">
-        <v>923862</v>
+        <v>913539</v>
       </c>
       <c r="Y41" s="8" t="n">
         <v>93</v>
       </c>
       <c r="BF41" s="9" t="n">
-        <v>28841</v>
+        <v>36047</v>
       </c>
       <c r="BG41" s="6" t="n">
-        <v>0.0112004013985259</v>
+        <v>0.01199583754720114</v>
       </c>
       <c r="BH41" s="10" t="n">
-        <v>2322980</v>
+        <v>2854115</v>
       </c>
       <c r="BI41" s="8" t="n">
-        <v>80.54436392635485</v>
+        <v>79.17760146475435</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>5100</t>
+          <t>5140</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Bonos Bernabo</t>
+          <t>Bonos Bagó</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>BERNABO</t>
+          <t>BAGO</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
@@ -3433,68 +3797,80 @@
         </is>
       </c>
       <c r="J42" s="5" t="n">
-        <v>4458</v>
+        <v>54581</v>
       </c>
       <c r="K42" s="6" t="n">
-        <v>0.004449004113682134</v>
+        <v>0.05491841876489149</v>
       </c>
       <c r="L42" s="7" t="n">
-        <v>329892</v>
+        <v>4038994</v>
       </c>
       <c r="M42" s="8" t="n">
         <v>74</v>
       </c>
       <c r="N42" s="5" t="n">
-        <v>4207</v>
+        <v>35663</v>
       </c>
       <c r="O42" s="6" t="n">
-        <v>0.005485871956332094</v>
+        <v>0.05167030569267302</v>
       </c>
       <c r="P42" s="7" t="n">
-        <v>311318</v>
+        <v>2639062</v>
       </c>
       <c r="Q42" s="8" t="n">
         <v>74</v>
       </c>
+      <c r="R42" s="5" t="n">
+        <v>29614</v>
+      </c>
+      <c r="S42" s="6" t="n">
+        <v>0.04378994312955991</v>
+      </c>
+      <c r="T42" s="7" t="n">
+        <v>2191436</v>
+      </c>
+      <c r="U42" s="8" t="n">
+        <v>74</v>
+      </c>
       <c r="V42" s="5" t="n">
-        <v>4464</v>
+        <v>15759</v>
       </c>
       <c r="W42" s="6" t="n">
-        <v>0.006831171812234592</v>
+        <v>0.0244467334547474</v>
       </c>
       <c r="X42" s="7" t="n">
-        <v>415152</v>
+        <v>1465587</v>
       </c>
       <c r="Y42" s="8" t="n">
         <v>93</v>
       </c>
       <c r="BF42" s="9" t="n">
-        <v>13129</v>
+        <v>135617</v>
       </c>
       <c r="BG42" s="6" t="n">
-        <v>0.005098646716869961</v>
+        <v>0.0451310650161949</v>
       </c>
       <c r="BH42" s="10" t="n">
-        <v>1056362</v>
+        <v>10335079</v>
       </c>
       <c r="BI42" s="8" t="n">
-        <v>80.46020260492041</v>
+        <v>76.20784267459095</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>5110</t>
+          <t>5150</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Bonos Eurolab</t>
+          <t>Bonos Caviahue</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>EUROLAB</t>
+          <t>CAVIAHUE</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
@@ -3528,68 +3904,80 @@
         </is>
       </c>
       <c r="J43" s="5" t="n">
-        <v>26534</v>
+        <v>1002</v>
       </c>
       <c r="K43" s="6" t="n">
-        <v>0.02648045651692278</v>
+        <v>0.001008194346062206</v>
       </c>
       <c r="L43" s="7" t="n">
-        <v>1963516</v>
+        <v>74148</v>
       </c>
       <c r="M43" s="8" t="n">
         <v>74</v>
       </c>
       <c r="N43" s="5" t="n">
-        <v>24819</v>
+        <v>982</v>
       </c>
       <c r="O43" s="6" t="n">
-        <v>0.03236364537299887</v>
+        <v>0.001422769822791266</v>
       </c>
       <c r="P43" s="7" t="n">
-        <v>1836606</v>
+        <v>72668</v>
       </c>
       <c r="Q43" s="8" t="n">
         <v>74</v>
       </c>
+      <c r="R43" s="5" t="n">
+        <v>804</v>
+      </c>
+      <c r="S43" s="6" t="n">
+        <v>0.001188867234286694</v>
+      </c>
+      <c r="T43" s="7" t="n">
+        <v>59496</v>
+      </c>
+      <c r="U43" s="8" t="n">
+        <v>74</v>
+      </c>
       <c r="V43" s="5" t="n">
-        <v>31434</v>
+        <v>2593</v>
       </c>
       <c r="W43" s="6" t="n">
-        <v>0.04810283484448525</v>
+        <v>0.004022487457843773</v>
       </c>
       <c r="X43" s="7" t="n">
-        <v>2923362</v>
+        <v>241149</v>
       </c>
       <c r="Y43" s="8" t="n">
         <v>93</v>
       </c>
       <c r="BF43" s="9" t="n">
-        <v>82787</v>
+        <v>5381</v>
       </c>
       <c r="BG43" s="6" t="n">
-        <v>0.03215032871882958</v>
+        <v>0.001790706628609575</v>
       </c>
       <c r="BH43" s="10" t="n">
-        <v>6723484</v>
+        <v>447461</v>
       </c>
       <c r="BI43" s="8" t="n">
-        <v>81.21424861391282</v>
+        <v>83.155733135105</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>5120</t>
+          <t>5160</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Eximia Cepage (Ceoderma) - vía Avanter</t>
+          <t>Bonos By Derm</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>CEODERMA</t>
+          <t>BYDERM</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
@@ -3604,7 +3992,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>SI - ETICOS</t>
+          <t>SI - DINAMICAS - BONOS</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -3623,44 +4011,80 @@
         </is>
       </c>
       <c r="J44" s="5" t="n">
-        <v>355</v>
+        <v>5461</v>
       </c>
       <c r="K44" s="6" t="n">
-        <v>0.0003542836384829874</v>
+        <v>0.005494759804237233</v>
       </c>
       <c r="L44" s="7" t="n">
-        <v>26270</v>
+        <v>404114</v>
       </c>
       <c r="M44" s="8" t="n">
         <v>74</v>
       </c>
+      <c r="N44" s="5" t="n">
+        <v>5116</v>
+      </c>
+      <c r="O44" s="6" t="n">
+        <v>0.007412312029939018</v>
+      </c>
+      <c r="P44" s="7" t="n">
+        <v>378584</v>
+      </c>
+      <c r="Q44" s="8" t="n">
+        <v>74</v>
+      </c>
+      <c r="R44" s="5" t="n">
+        <v>6240</v>
+      </c>
+      <c r="S44" s="6" t="n">
+        <v>0.009227029281031061</v>
+      </c>
+      <c r="T44" s="7" t="n">
+        <v>461760</v>
+      </c>
+      <c r="U44" s="8" t="n">
+        <v>74</v>
+      </c>
+      <c r="V44" s="5" t="n">
+        <v>6100</v>
+      </c>
+      <c r="W44" s="6" t="n">
+        <v>0.009462851327746631</v>
+      </c>
+      <c r="X44" s="7" t="n">
+        <v>567300</v>
+      </c>
+      <c r="Y44" s="8" t="n">
+        <v>93</v>
+      </c>
       <c r="BF44" s="9" t="n">
-        <v>355</v>
+        <v>22917</v>
       </c>
       <c r="BG44" s="6" t="n">
-        <v>0.000137864238288433</v>
+        <v>0.007626393571426432</v>
       </c>
       <c r="BH44" s="10" t="n">
-        <v>26270</v>
+        <v>1811758</v>
       </c>
       <c r="BI44" s="8" t="n">
-        <v>74</v>
+        <v>79.05738098354934</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>5130</t>
+          <t>5170</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Bonos Cassara</t>
+          <t>Bonos Bioderma</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>CASSARA</t>
+          <t>BIODERMA</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
@@ -3694,68 +4118,80 @@
         </is>
       </c>
       <c r="J45" s="5" t="n">
-        <v>8603</v>
+        <v>1129</v>
       </c>
       <c r="K45" s="6" t="n">
-        <v>0.0085856398362511</v>
+        <v>0.001135979457788653</v>
       </c>
       <c r="L45" s="7" t="n">
-        <v>636622</v>
+        <v>83546</v>
       </c>
       <c r="M45" s="8" t="n">
         <v>74</v>
       </c>
       <c r="N45" s="5" t="n">
-        <v>7894</v>
+        <v>1053</v>
       </c>
       <c r="O45" s="6" t="n">
-        <v>0.0102936708398587</v>
+        <v>0.001525638109367824</v>
       </c>
       <c r="P45" s="7" t="n">
-        <v>584156</v>
+        <v>77922</v>
       </c>
       <c r="Q45" s="8" t="n">
         <v>74</v>
       </c>
+      <c r="R45" s="5" t="n">
+        <v>1289</v>
+      </c>
+      <c r="S45" s="6" t="n">
+        <v>0.001906032170392474</v>
+      </c>
+      <c r="T45" s="7" t="n">
+        <v>95386</v>
+      </c>
+      <c r="U45" s="8" t="n">
+        <v>74</v>
+      </c>
       <c r="V45" s="5" t="n">
-        <v>9823</v>
+        <v>1462</v>
       </c>
       <c r="W45" s="6" t="n">
-        <v>0.01503194460384866</v>
+        <v>0.002267981744453373</v>
       </c>
       <c r="X45" s="7" t="n">
-        <v>913539</v>
+        <v>135966</v>
       </c>
       <c r="Y45" s="8" t="n">
         <v>93</v>
       </c>
       <c r="BF45" s="9" t="n">
-        <v>26320</v>
+        <v>4933</v>
       </c>
       <c r="BG45" s="6" t="n">
-        <v>0.01022137113169452</v>
+        <v>0.001641619735909874</v>
       </c>
       <c r="BH45" s="10" t="n">
-        <v>2134317</v>
+        <v>392820</v>
       </c>
       <c r="BI45" s="8" t="n">
-        <v>81.09107142857142</v>
+        <v>79.63105615244274</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>5140</t>
+          <t>5180</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Bonos Bagó</t>
+          <t>Bonos Biferdil</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>BAGO</t>
+          <t>BIFERDIL</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
@@ -3785,72 +4221,84 @@
       </c>
       <c r="I46" s="4" t="inlineStr">
         <is>
-          <t>PRODUCTIVO</t>
+          <t>STARTUP</t>
         </is>
       </c>
       <c r="J46" s="5" t="n">
-        <v>54581</v>
+        <v>10</v>
       </c>
       <c r="K46" s="6" t="n">
-        <v>0.05447085992123925</v>
+        <v>1.00618198209801e-05</v>
       </c>
       <c r="L46" s="7" t="n">
-        <v>4038994</v>
+        <v>740</v>
       </c>
       <c r="M46" s="8" t="n">
         <v>74</v>
       </c>
       <c r="N46" s="5" t="n">
-        <v>35663</v>
+        <v>12</v>
       </c>
       <c r="O46" s="6" t="n">
-        <v>0.04650407691435024</v>
+        <v>1.7386189280545e-05</v>
       </c>
       <c r="P46" s="7" t="n">
-        <v>2639062</v>
+        <v>888</v>
       </c>
       <c r="Q46" s="8" t="n">
         <v>74</v>
       </c>
+      <c r="R46" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="S46" s="6" t="n">
+        <v>2.070166825872353e-05</v>
+      </c>
+      <c r="T46" s="7" t="n">
+        <v>1036</v>
+      </c>
+      <c r="U46" s="8" t="n">
+        <v>74</v>
+      </c>
       <c r="V46" s="5" t="n">
-        <v>15759</v>
+        <v>22</v>
       </c>
       <c r="W46" s="6" t="n">
-        <v>0.02411568920004591</v>
+        <v>3.412831626400425e-05</v>
       </c>
       <c r="X46" s="7" t="n">
-        <v>1465587</v>
+        <v>2046</v>
       </c>
       <c r="Y46" s="8" t="n">
         <v>93</v>
       </c>
       <c r="BF46" s="9" t="n">
-        <v>106003</v>
+        <v>58</v>
       </c>
       <c r="BG46" s="6" t="n">
-        <v>0.04116626155292608</v>
+        <v>1.930142807272911e-05</v>
       </c>
       <c r="BH46" s="10" t="n">
-        <v>8143643</v>
+        <v>4710</v>
       </c>
       <c r="BI46" s="8" t="n">
-        <v>76.82464647226965</v>
+        <v>81.20689655172414</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>5150</t>
+          <t>5190</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Bonos Caviahue</t>
+          <t>Bonos Fresenius</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>CAVIAHUE</t>
+          <t>FRESENIUS</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
@@ -3880,72 +4328,84 @@
       </c>
       <c r="I47" s="4" t="inlineStr">
         <is>
-          <t>PRODUCTIVO</t>
+          <t>STARTUP</t>
         </is>
       </c>
       <c r="J47" s="5" t="n">
-        <v>1002</v>
+        <v>47</v>
       </c>
       <c r="K47" s="6" t="n">
-        <v>0.0009999780443942349</v>
+        <v>4.729055315860648e-05</v>
       </c>
       <c r="L47" s="7" t="n">
-        <v>74148</v>
+        <v>3478</v>
       </c>
       <c r="M47" s="8" t="n">
         <v>74</v>
       </c>
       <c r="N47" s="5" t="n">
-        <v>982</v>
+        <v>38</v>
       </c>
       <c r="O47" s="6" t="n">
-        <v>0.001280514918259595</v>
+        <v>5.505626605505916e-05</v>
       </c>
       <c r="P47" s="7" t="n">
-        <v>72668</v>
+        <v>2812</v>
       </c>
       <c r="Q47" s="8" t="n">
         <v>74</v>
       </c>
+      <c r="R47" s="5" t="n">
+        <v>46</v>
+      </c>
+      <c r="S47" s="6" t="n">
+        <v>6.80197671358059e-05</v>
+      </c>
+      <c r="T47" s="7" t="n">
+        <v>3404</v>
+      </c>
+      <c r="U47" s="8" t="n">
+        <v>74</v>
+      </c>
       <c r="V47" s="5" t="n">
-        <v>2593</v>
+        <v>107</v>
       </c>
       <c r="W47" s="6" t="n">
-        <v>0.003968017139140747</v>
+        <v>0.0001659877200112934</v>
       </c>
       <c r="X47" s="7" t="n">
-        <v>241149</v>
+        <v>9951</v>
       </c>
       <c r="Y47" s="8" t="n">
         <v>93</v>
       </c>
       <c r="BF47" s="9" t="n">
-        <v>4577</v>
+        <v>238</v>
       </c>
       <c r="BG47" s="6" t="n">
-        <v>0.001777477799003261</v>
+        <v>7.920241174671601e-05</v>
       </c>
       <c r="BH47" s="10" t="n">
-        <v>387965</v>
+        <v>19645</v>
       </c>
       <c r="BI47" s="8" t="n">
-        <v>84.76403757920035</v>
+        <v>82.54201680672269</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>5160</t>
+          <t>5200</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Bonos By Derm</t>
+          <t>Bonos SC Johnson</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>BYDERM</t>
+          <t>SC JHONSON</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
@@ -3975,72 +4435,84 @@
       </c>
       <c r="I48" s="4" t="inlineStr">
         <is>
-          <t>PRODUCTIVO</t>
+          <t>STARTUP</t>
         </is>
       </c>
       <c r="J48" s="5" t="n">
-        <v>5461</v>
+        <v>16</v>
       </c>
       <c r="K48" s="6" t="n">
-        <v>0.005449980140156603</v>
+        <v>1.609891171356816e-05</v>
       </c>
       <c r="L48" s="7" t="n">
-        <v>404114</v>
+        <v>1184</v>
       </c>
       <c r="M48" s="8" t="n">
         <v>74</v>
       </c>
       <c r="N48" s="5" t="n">
-        <v>5116</v>
+        <v>20</v>
       </c>
       <c r="O48" s="6" t="n">
-        <v>0.006671195847063226</v>
+        <v>2.897698213424167e-05</v>
       </c>
       <c r="P48" s="7" t="n">
-        <v>378584</v>
+        <v>1480</v>
       </c>
       <c r="Q48" s="8" t="n">
         <v>74</v>
       </c>
+      <c r="R48" s="5" t="n">
+        <v>24</v>
+      </c>
+      <c r="S48" s="6" t="n">
+        <v>3.548857415781177e-05</v>
+      </c>
+      <c r="T48" s="7" t="n">
+        <v>1776</v>
+      </c>
+      <c r="U48" s="8" t="n">
+        <v>74</v>
+      </c>
       <c r="V48" s="5" t="n">
-        <v>6100</v>
+        <v>6</v>
       </c>
       <c r="W48" s="6" t="n">
-        <v>0.009334710585714832</v>
+        <v>9.307722617455703e-06</v>
       </c>
       <c r="X48" s="7" t="n">
-        <v>567300</v>
+        <v>558</v>
       </c>
       <c r="Y48" s="8" t="n">
         <v>93</v>
       </c>
       <c r="BF48" s="9" t="n">
-        <v>16677</v>
+        <v>66</v>
       </c>
       <c r="BG48" s="6" t="n">
-        <v>0.006476512399820272</v>
+        <v>2.19636940137952e-05</v>
       </c>
       <c r="BH48" s="10" t="n">
-        <v>1349998</v>
+        <v>4998</v>
       </c>
       <c r="BI48" s="8" t="n">
-        <v>80.9496911914613</v>
+        <v>75.72727272727273</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>5170</t>
+          <t>5210</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Bonos Bioderma</t>
+          <t>Bonos Pharmatrix</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>BIODERMA</t>
+          <t>PHARMATRIX</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
@@ -4070,72 +4542,84 @@
       </c>
       <c r="I49" s="4" t="inlineStr">
         <is>
-          <t>PRODUCTIVO</t>
+          <t>STARTUP</t>
         </is>
       </c>
       <c r="J49" s="5" t="n">
-        <v>1129</v>
+        <v>85</v>
       </c>
       <c r="K49" s="6" t="n">
-        <v>0.001126721768583923</v>
+        <v>8.552546847833087e-05</v>
       </c>
       <c r="L49" s="7" t="n">
-        <v>83546</v>
+        <v>6290</v>
       </c>
       <c r="M49" s="8" t="n">
         <v>74</v>
       </c>
       <c r="N49" s="5" t="n">
-        <v>1053</v>
+        <v>80</v>
       </c>
       <c r="O49" s="6" t="n">
-        <v>0.001373097972431114</v>
+        <v>0.0001159079285369667</v>
       </c>
       <c r="P49" s="7" t="n">
-        <v>77922</v>
+        <v>5920</v>
       </c>
       <c r="Q49" s="8" t="n">
         <v>74</v>
       </c>
+      <c r="R49" s="5" t="n">
+        <v>248</v>
+      </c>
+      <c r="S49" s="6" t="n">
+        <v>0.0003667152662973883</v>
+      </c>
+      <c r="T49" s="7" t="n">
+        <v>18352</v>
+      </c>
+      <c r="U49" s="8" t="n">
+        <v>74</v>
+      </c>
       <c r="V49" s="5" t="n">
-        <v>1462</v>
+        <v>320</v>
       </c>
       <c r="W49" s="6" t="n">
-        <v>0.002237269979723784</v>
+        <v>0.0004964118729309709</v>
       </c>
       <c r="X49" s="7" t="n">
-        <v>135966</v>
+        <v>29760</v>
       </c>
       <c r="Y49" s="8" t="n">
         <v>93</v>
       </c>
       <c r="BF49" s="9" t="n">
-        <v>3644</v>
+        <v>733</v>
       </c>
       <c r="BG49" s="6" t="n">
-        <v>0.001415147279783239</v>
+        <v>0.00024393011685018</v>
       </c>
       <c r="BH49" s="10" t="n">
-        <v>297434</v>
+        <v>60322</v>
       </c>
       <c r="BI49" s="8" t="n">
-        <v>81.62294182217343</v>
+        <v>82.29467939972714</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>5180</t>
+          <t>5220</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Bonos Biferdil</t>
+          <t>Bonos Megalabs</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>BIFERDIL</t>
+          <t>MEGALABS</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
@@ -4169,68 +4653,47 @@
         </is>
       </c>
       <c r="J50" s="5" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="K50" s="6" t="n">
-        <v>9.979820802337674e-06</v>
+        <v>0</v>
       </c>
       <c r="L50" s="7" t="n">
-        <v>740</v>
-      </c>
-      <c r="M50" s="8" t="n">
-        <v>74</v>
+        <v>0</v>
       </c>
       <c r="N50" s="5" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="O50" s="6" t="n">
-        <v>1.564784014166511e-05</v>
+        <v>0</v>
       </c>
       <c r="P50" s="7" t="n">
-        <v>888</v>
-      </c>
-      <c r="Q50" s="8" t="n">
-        <v>74</v>
-      </c>
-      <c r="V50" s="5" t="n">
-        <v>22</v>
-      </c>
-      <c r="W50" s="6" t="n">
-        <v>3.366616932552891e-05</v>
-      </c>
-      <c r="X50" s="7" t="n">
-        <v>2046</v>
-      </c>
-      <c r="Y50" s="8" t="n">
-        <v>93</v>
-      </c>
-      <c r="BF50" s="9" t="n">
-        <v>44</v>
-      </c>
-      <c r="BG50" s="6" t="n">
-        <v>1.708739854842549e-05</v>
-      </c>
-      <c r="BH50" s="10" t="n">
-        <v>3674</v>
-      </c>
-      <c r="BI50" s="8" t="n">
-        <v>83.5</v>
+        <v>0</v>
+      </c>
+      <c r="R50" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S50" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T50" s="7" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>5190</t>
+          <t>5230</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Bonos Fresenius</t>
+          <t>Bonos Siegfried</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>FRESENIUS</t>
+          <t>SIEGFRIED</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
@@ -4264,68 +4727,29 @@
         </is>
       </c>
       <c r="J51" s="5" t="n">
-        <v>47</v>
+        <v>0</v>
       </c>
       <c r="K51" s="6" t="n">
-        <v>4.690515777098706e-05</v>
+        <v>0</v>
       </c>
       <c r="L51" s="7" t="n">
-        <v>3478</v>
-      </c>
-      <c r="M51" s="8" t="n">
-        <v>74</v>
-      </c>
-      <c r="N51" s="5" t="n">
-        <v>38</v>
-      </c>
-      <c r="O51" s="6" t="n">
-        <v>4.955149378193952e-05</v>
-      </c>
-      <c r="P51" s="7" t="n">
-        <v>2812</v>
-      </c>
-      <c r="Q51" s="8" t="n">
-        <v>74</v>
-      </c>
-      <c r="V51" s="5" t="n">
-        <v>107</v>
-      </c>
-      <c r="W51" s="6" t="n">
-        <v>0.0001637400053559815</v>
-      </c>
-      <c r="X51" s="7" t="n">
-        <v>9951</v>
-      </c>
-      <c r="Y51" s="8" t="n">
-        <v>93</v>
-      </c>
-      <c r="BF51" s="9" t="n">
-        <v>192</v>
-      </c>
-      <c r="BG51" s="6" t="n">
-        <v>7.456319366585669e-05</v>
-      </c>
-      <c r="BH51" s="10" t="n">
-        <v>16241</v>
-      </c>
-      <c r="BI51" s="8" t="n">
-        <v>84.58854166666667</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>5200</t>
+          <t>5240</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Bonos SC Johnson</t>
+          <t>Bonos Raisse</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>SC JHONSON</t>
+          <t>RAISSE</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
@@ -4359,68 +4783,56 @@
         </is>
       </c>
       <c r="J52" s="5" t="n">
-        <v>16</v>
+        <v>167</v>
       </c>
       <c r="K52" s="6" t="n">
-        <v>1.596771328374028e-05</v>
+        <v>0.0001680323910103677</v>
       </c>
       <c r="L52" s="7" t="n">
-        <v>1184</v>
+        <v>12358</v>
       </c>
       <c r="M52" s="8" t="n">
         <v>74</v>
       </c>
       <c r="N52" s="5" t="n">
-        <v>20</v>
+        <v>356</v>
       </c>
       <c r="O52" s="6" t="n">
-        <v>2.607973356944185e-05</v>
+        <v>0.0005157902819895016</v>
       </c>
       <c r="P52" s="7" t="n">
-        <v>1480</v>
+        <v>26344</v>
       </c>
       <c r="Q52" s="8" t="n">
         <v>74</v>
       </c>
-      <c r="V52" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="W52" s="6" t="n">
-        <v>9.181682543326065e-06</v>
-      </c>
-      <c r="X52" s="7" t="n">
-        <v>558</v>
-      </c>
-      <c r="Y52" s="8" t="n">
-        <v>93</v>
-      </c>
       <c r="BF52" s="9" t="n">
-        <v>42</v>
+        <v>523</v>
       </c>
       <c r="BG52" s="6" t="n">
-        <v>1.631069861440615e-05</v>
+        <v>0.0001740456358971953</v>
       </c>
       <c r="BH52" s="10" t="n">
-        <v>3222</v>
+        <v>38702</v>
       </c>
       <c r="BI52" s="8" t="n">
-        <v>76.71428571428571</v>
+        <v>74</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>5210</t>
+          <t>5250</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Bonos Pharmatrix</t>
+          <t>Bonos Siscom (Rayito de Sol)</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>PHARMATRIX</t>
+          <t>SISCOM</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
@@ -4454,68 +4866,62 @@
         </is>
       </c>
       <c r="J53" s="5" t="n">
-        <v>85</v>
+        <v>0</v>
       </c>
       <c r="K53" s="6" t="n">
-        <v>8.482847681987022e-05</v>
+        <v>0</v>
       </c>
       <c r="L53" s="7" t="n">
-        <v>6290</v>
-      </c>
-      <c r="M53" s="8" t="n">
-        <v>74</v>
+        <v>0</v>
       </c>
       <c r="N53" s="5" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="O53" s="6" t="n">
-        <v>0.0001043189342777674</v>
+        <v>0</v>
       </c>
       <c r="P53" s="7" t="n">
-        <v>5920</v>
-      </c>
-      <c r="Q53" s="8" t="n">
-        <v>74</v>
+        <v>0</v>
       </c>
       <c r="V53" s="5" t="n">
-        <v>320</v>
+        <v>1</v>
       </c>
       <c r="W53" s="6" t="n">
-        <v>0.0004896897356440568</v>
+        <v>1.551287102909284e-06</v>
       </c>
       <c r="X53" s="7" t="n">
-        <v>29760</v>
+        <v>93</v>
       </c>
       <c r="Y53" s="8" t="n">
         <v>93</v>
       </c>
       <c r="BF53" s="9" t="n">
-        <v>485</v>
+        <v>1</v>
       </c>
       <c r="BG53" s="6" t="n">
-        <v>0.0001883497339996901</v>
+        <v>3.327832426332606e-07</v>
       </c>
       <c r="BH53" s="10" t="n">
-        <v>41970</v>
+        <v>93</v>
       </c>
       <c r="BI53" s="8" t="n">
-        <v>86.5360824742268</v>
+        <v>93</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>5220</t>
+          <t>5260</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Bonos Megalabs</t>
+          <t>Bonos ENA (alta 22/04/2026)</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>MEGALABS</t>
+          <t>ENA</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
@@ -4528,19 +4934,15 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>SI - DINAMICAS - BONOS</t>
-        </is>
-      </c>
+      <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Facturado vía Avanter - valor unitario por TRX</t>
+          <t>Alta laboratorio nuevo - Avanter</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>Trimestral por IPC Indec</t>
+          <t>Mensual</t>
         </is>
       </c>
       <c r="I54" s="4" t="inlineStr">
@@ -4548,39 +4950,27 @@
           <t>STARTUP</t>
         </is>
       </c>
-      <c r="J54" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K54" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L54" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N54" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O54" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="P54" s="7" t="n">
-        <v>0</v>
+      <c r="X54" s="7" t="n">
+        <v>547420.8</v>
+      </c>
+      <c r="BH54" s="10" t="n">
+        <v>547420.8</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>5230</t>
+          <t>5270</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Bonos Siegfried</t>
+          <t>Bonos Convatec (alta 24/04/2026)</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>SIEGFRIED</t>
+          <t>CONVATEC</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
@@ -4593,19 +4983,15 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>SI - DINAMICAS - BONOS</t>
-        </is>
-      </c>
+      <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Facturado vía Avanter - valor unitario por TRX</t>
+          <t>Alta laboratorio nuevo - Avanter</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>Trimestral por IPC Indec</t>
+          <t>Mensual</t>
         </is>
       </c>
       <c r="I55" s="4" t="inlineStr">
@@ -4613,368 +4999,95 @@
           <t>STARTUP</t>
         </is>
       </c>
-      <c r="J55" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K55" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L55" s="7" t="n">
-        <v>0</v>
+      <c r="X55" s="7" t="n">
+        <v>547420.8</v>
+      </c>
+      <c r="BH55" s="10" t="n">
+        <v>547420.8</v>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="4" t="inlineStr">
-        <is>
-          <t>5240</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>Bonos Raisse</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>RAISSE</t>
-        </is>
-      </c>
-      <c r="D56" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E56" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>SI - DINAMICAS - BONOS</t>
-        </is>
-      </c>
-      <c r="G56" t="inlineStr">
-        <is>
-          <t>Facturado vía Avanter - valor unitario por TRX</t>
-        </is>
-      </c>
-      <c r="H56" t="inlineStr">
-        <is>
-          <t>Trimestral por IPC Indec</t>
-        </is>
-      </c>
-      <c r="I56" s="4" t="inlineStr">
-        <is>
-          <t>STARTUP</t>
-        </is>
-      </c>
-      <c r="J56" s="5" t="n">
-        <v>167</v>
-      </c>
-      <c r="K56" s="6" t="n">
-        <v>0.0001666630073990391</v>
-      </c>
-      <c r="L56" s="7" t="n">
-        <v>12358</v>
-      </c>
-      <c r="M56" s="8" t="n">
-        <v>74</v>
-      </c>
-      <c r="N56" s="5" t="n">
-        <v>356</v>
-      </c>
-      <c r="O56" s="6" t="n">
-        <v>0.000464219257536065</v>
-      </c>
-      <c r="P56" s="7" t="n">
-        <v>26344</v>
-      </c>
-      <c r="Q56" s="8" t="n">
-        <v>74</v>
-      </c>
-      <c r="BF56" s="9" t="n">
-        <v>523</v>
-      </c>
-      <c r="BG56" s="6" t="n">
-        <v>0.0002031070327460576</v>
-      </c>
-      <c r="BH56" s="10" t="n">
-        <v>38702</v>
-      </c>
-      <c r="BI56" s="8" t="n">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="4" t="inlineStr">
-        <is>
-          <t>5250</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>Bonos Siscom (Rayito de Sol)</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>SISCOM</t>
-        </is>
-      </c>
-      <c r="D57" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E57" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="F57" t="inlineStr">
-        <is>
-          <t>SI - DINAMICAS - BONOS</t>
-        </is>
-      </c>
-      <c r="G57" t="inlineStr">
-        <is>
-          <t>Facturado vía Avanter - valor unitario por TRX</t>
-        </is>
-      </c>
-      <c r="H57" t="inlineStr">
-        <is>
-          <t>Trimestral por IPC Indec</t>
-        </is>
-      </c>
-      <c r="I57" s="4" t="inlineStr">
-        <is>
-          <t>STARTUP</t>
-        </is>
-      </c>
-      <c r="J57" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K57" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L57" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N57" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O57" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="P57" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="V57" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="W57" s="6" t="n">
-        <v>1.530280423887677e-06</v>
-      </c>
-      <c r="X57" s="7" t="n">
-        <v>93</v>
-      </c>
-      <c r="Y57" s="8" t="n">
-        <v>93</v>
-      </c>
-      <c r="BF57" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="BG57" s="6" t="n">
-        <v>3.883499670096703e-07</v>
-      </c>
-      <c r="BH57" s="10" t="n">
-        <v>93</v>
-      </c>
-      <c r="BI57" s="8" t="n">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="4" t="inlineStr">
-        <is>
-          <t>5260</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>Bonos ENA (alta 22/04/2026)</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>ENA</t>
-        </is>
-      </c>
-      <c r="D58" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E58" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr"/>
-      <c r="G58" t="inlineStr">
-        <is>
-          <t>Alta laboratorio nuevo - Avanter</t>
-        </is>
-      </c>
-      <c r="H58" t="inlineStr">
-        <is>
-          <t>Mensual</t>
-        </is>
-      </c>
-      <c r="I58" s="4" t="inlineStr">
-        <is>
-          <t>STARTUP</t>
-        </is>
-      </c>
-      <c r="X58" s="7" t="n">
-        <v>547420.8</v>
-      </c>
-      <c r="BH58" s="10" t="n">
-        <v>547420.8</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="4" t="inlineStr">
-        <is>
-          <t>5270</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>Bonos Convatec (alta 24/04/2026)</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>CONVATEC</t>
-        </is>
-      </c>
-      <c r="D59" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E59" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr"/>
-      <c r="G59" t="inlineStr">
-        <is>
-          <t>Alta laboratorio nuevo - Avanter</t>
-        </is>
-      </c>
-      <c r="H59" t="inlineStr">
-        <is>
-          <t>Mensual</t>
-        </is>
-      </c>
-      <c r="I59" s="4" t="inlineStr">
-        <is>
-          <t>STARTUP</t>
-        </is>
-      </c>
-      <c r="X59" s="7" t="n">
-        <v>547420.8</v>
-      </c>
-      <c r="BH59" s="10" t="n">
-        <v>547420.8</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="11" t="inlineStr">
+      <c r="A56" s="11" t="inlineStr">
         <is>
           <t>TOTAL GENERAL</t>
         </is>
       </c>
-      <c r="J60" s="12" t="n">
-        <v>1002022</v>
-      </c>
-      <c r="K60" s="13" t="n"/>
-      <c r="L60" s="14" t="n">
-        <v>89706119.75</v>
-      </c>
-      <c r="M60" s="13" t="n"/>
-      <c r="N60" s="12" t="n">
-        <v>766879</v>
-      </c>
-      <c r="O60" s="13" t="n"/>
-      <c r="P60" s="14" t="n">
-        <v>69228656.50999999</v>
-      </c>
-      <c r="Q60" s="13" t="n"/>
-      <c r="R60" s="12" t="n">
-        <v>152621</v>
-      </c>
-      <c r="S60" s="13" t="n"/>
-      <c r="T60" s="14" t="n">
-        <v>29259222.98</v>
-      </c>
-      <c r="U60" s="13" t="n"/>
-      <c r="V60" s="12" t="n">
-        <v>653475</v>
-      </c>
-      <c r="W60" s="13" t="n"/>
-      <c r="X60" s="14" t="n">
-        <v>80417563.47999999</v>
-      </c>
-      <c r="Y60" s="13" t="n"/>
-      <c r="Z60" s="12" t="n"/>
-      <c r="AA60" s="13" t="n"/>
-      <c r="AB60" s="14" t="n"/>
-      <c r="AC60" s="13" t="n"/>
-      <c r="AD60" s="12" t="n"/>
-      <c r="AE60" s="13" t="n"/>
-      <c r="AF60" s="14" t="n"/>
-      <c r="AG60" s="13" t="n"/>
-      <c r="AH60" s="12" t="n"/>
-      <c r="AI60" s="13" t="n"/>
-      <c r="AJ60" s="14" t="n"/>
-      <c r="AK60" s="13" t="n"/>
-      <c r="AL60" s="12" t="n"/>
-      <c r="AM60" s="13" t="n"/>
-      <c r="AN60" s="14" t="n"/>
-      <c r="AO60" s="13" t="n"/>
-      <c r="AP60" s="12" t="n"/>
-      <c r="AQ60" s="13" t="n"/>
-      <c r="AR60" s="14" t="n"/>
-      <c r="AS60" s="13" t="n"/>
-      <c r="AT60" s="12" t="n"/>
-      <c r="AU60" s="13" t="n"/>
-      <c r="AV60" s="14" t="n"/>
-      <c r="AW60" s="13" t="n"/>
-      <c r="AX60" s="12" t="n"/>
-      <c r="AY60" s="13" t="n"/>
-      <c r="AZ60" s="14" t="n"/>
-      <c r="BA60" s="13" t="n"/>
-      <c r="BB60" s="12" t="n"/>
-      <c r="BC60" s="13" t="n"/>
-      <c r="BD60" s="14" t="n"/>
-      <c r="BE60" s="13" t="n"/>
-      <c r="BF60" s="12" t="n">
-        <v>2574997</v>
-      </c>
-      <c r="BG60" s="13" t="n"/>
-      <c r="BH60" s="14" t="n">
-        <v>268611562.72</v>
-      </c>
-      <c r="BI60" s="13" t="n"/>
+      <c r="J56" s="12" t="n">
+        <v>993856</v>
+      </c>
+      <c r="K56" s="13" t="n"/>
+      <c r="L56" s="14" t="n">
+        <v>88632610.45</v>
+      </c>
+      <c r="M56" s="13" t="n"/>
+      <c r="N56" s="12" t="n">
+        <v>690203</v>
+      </c>
+      <c r="O56" s="13" t="n"/>
+      <c r="P56" s="14" t="n">
+        <v>64684069.98999999</v>
+      </c>
+      <c r="Q56" s="13" t="n"/>
+      <c r="R56" s="12" t="n">
+        <v>676274</v>
+      </c>
+      <c r="S56" s="13" t="n"/>
+      <c r="T56" s="14" t="n">
+        <v>67359067</v>
+      </c>
+      <c r="U56" s="13" t="n"/>
+      <c r="V56" s="12" t="n">
+        <v>644626</v>
+      </c>
+      <c r="W56" s="13" t="n"/>
+      <c r="X56" s="14" t="n">
+        <v>78946556.27</v>
+      </c>
+      <c r="Y56" s="13" t="n"/>
+      <c r="Z56" s="12" t="n"/>
+      <c r="AA56" s="13" t="n"/>
+      <c r="AB56" s="14" t="n"/>
+      <c r="AC56" s="13" t="n"/>
+      <c r="AD56" s="12" t="n"/>
+      <c r="AE56" s="13" t="n"/>
+      <c r="AF56" s="14" t="n"/>
+      <c r="AG56" s="13" t="n"/>
+      <c r="AH56" s="12" t="n"/>
+      <c r="AI56" s="13" t="n"/>
+      <c r="AJ56" s="14" t="n"/>
+      <c r="AK56" s="13" t="n"/>
+      <c r="AL56" s="12" t="n"/>
+      <c r="AM56" s="13" t="n"/>
+      <c r="AN56" s="14" t="n"/>
+      <c r="AO56" s="13" t="n"/>
+      <c r="AP56" s="12" t="n"/>
+      <c r="AQ56" s="13" t="n"/>
+      <c r="AR56" s="14" t="n"/>
+      <c r="AS56" s="13" t="n"/>
+      <c r="AT56" s="12" t="n"/>
+      <c r="AU56" s="13" t="n"/>
+      <c r="AV56" s="14" t="n"/>
+      <c r="AW56" s="13" t="n"/>
+      <c r="AX56" s="12" t="n"/>
+      <c r="AY56" s="13" t="n"/>
+      <c r="AZ56" s="14" t="n"/>
+      <c r="BA56" s="13" t="n"/>
+      <c r="BB56" s="12" t="n"/>
+      <c r="BC56" s="13" t="n"/>
+      <c r="BD56" s="14" t="n"/>
+      <c r="BE56" s="13" t="n"/>
+      <c r="BF56" s="12" t="n">
+        <v>3004959</v>
+      </c>
+      <c r="BG56" s="13" t="n"/>
+      <c r="BH56" s="14" t="n">
+        <v>299622303.71</v>
+      </c>
+      <c r="BI56" s="13" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="27">
-    <mergeCell ref="A27:BI27"/>
+  <mergeCells count="25">
+    <mergeCell ref="A56:I56"/>
     <mergeCell ref="A3:BI3"/>
     <mergeCell ref="A21:BI21"/>
     <mergeCell ref="Z1:AC1"/>
@@ -4986,7 +5099,6 @@
     <mergeCell ref="A17:BI17"/>
     <mergeCell ref="A23:BI23"/>
     <mergeCell ref="AX1:BA1"/>
-    <mergeCell ref="A29:BI29"/>
     <mergeCell ref="J1:M1"/>
     <mergeCell ref="A19:BI19"/>
     <mergeCell ref="A10:BI10"/>
@@ -4996,7 +5108,6 @@
     <mergeCell ref="AD1:AG1"/>
     <mergeCell ref="AP1:AS1"/>
     <mergeCell ref="AH1:AK1"/>
-    <mergeCell ref="A60:I60"/>
     <mergeCell ref="N1:Q1"/>
     <mergeCell ref="BB1:BE1"/>
     <mergeCell ref="A7:BI7"/>
@@ -5012,7 +5123,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -5069,19 +5180,19 @@
         </is>
       </c>
       <c r="B4" s="8" t="n">
-        <v>198.48</v>
+        <v>203.33</v>
       </c>
       <c r="C4" s="8" t="n">
-        <v>138.74</v>
+        <v>198.11</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>191.71</v>
+        <v>194.3</v>
       </c>
       <c r="E4" s="8" t="n">
-        <v>199.46</v>
+        <v>201.34</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>179.74</v>
+        <v>199.17</v>
       </c>
     </row>
     <row r="5">
@@ -5096,11 +5207,14 @@
       <c r="C5" s="8" t="n">
         <v>74</v>
       </c>
+      <c r="D5" s="8" t="n">
+        <v>74</v>
+      </c>
       <c r="E5" s="8" t="n">
         <v>93</v>
       </c>
       <c r="F5" s="8" t="n">
-        <v>78.73999999999999</v>
+        <v>77.73</v>
       </c>
     </row>
     <row r="7">
@@ -5260,40 +5374,14 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>PROVINCIA ART (nuevo 2026)</t>
+          <t>AVANTER</t>
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>25707</v>
+        <v>2489174</v>
       </c>
       <c r="C19" s="7" t="n">
-        <v>3838202.49</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>SERDATA (nuevo 2026)</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="n">
-        <v>76676</v>
-      </c>
-      <c r="C20" s="7" t="n">
-        <v>4544586.52</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>AVANTER</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="n">
-        <v>1956829</v>
-      </c>
-      <c r="C21" s="7" t="n">
-        <v>155175740.6</v>
+        <v>194569270.6</v>
       </c>
     </row>
   </sheetData>
@@ -5417,7 +5505,7 @@
         </is>
       </c>
       <c r="B3" s="8" t="n">
-        <v>179.74</v>
+        <v>199.17</v>
       </c>
     </row>
     <row r="4">
@@ -5427,7 +5515,7 @@
         </is>
       </c>
       <c r="B4" s="8" t="n">
-        <v>78.73999999999999</v>
+        <v>77.73</v>
       </c>
     </row>
   </sheetData>
@@ -5441,7 +5529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B45"/>
+  <dimension ref="A1:B43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5467,7 +5555,7 @@
         </is>
       </c>
       <c r="B2" s="5" t="n">
-        <v>1151690</v>
+        <v>1425880</v>
       </c>
     </row>
     <row r="3">
@@ -5487,27 +5575,27 @@
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>233291</v>
+        <v>308616</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>5140</t>
+          <t>5020</t>
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>106003</v>
+        <v>136340</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>5020</t>
+          <t>5140</t>
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>101736</v>
+        <v>135617</v>
       </c>
     </row>
     <row r="7">
@@ -5517,97 +5605,97 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>88671</v>
+        <v>116927</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>5060</t>
+          <t>5110</t>
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>84177</v>
+        <v>113488</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>5110</t>
+          <t>5060</t>
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>82787</v>
+        <v>105857</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>5320</t>
+          <t>5028</t>
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>76676</v>
+        <v>62353</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>5028</t>
+          <t>5005</t>
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>62353</v>
+        <v>58552</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>5005</t>
+          <t>5090</t>
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>58552</v>
+        <v>38929</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>5090</t>
+          <t>5130</t>
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>28841</v>
+        <v>36047</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>5130</t>
+          <t>5160</t>
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>26320</v>
+        <v>22917</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>5310</t>
+          <t>5025</t>
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>25707</v>
+        <v>18368</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>5025</t>
+          <t>5100</t>
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>18368</v>
+        <v>17738</v>
       </c>
     </row>
     <row r="17">
@@ -5623,51 +5711,51 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>5160</t>
+          <t>5040</t>
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>16677</v>
+        <v>12015</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>5100</t>
+          <t>5023</t>
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>13129</v>
+        <v>8151</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>5040</t>
+          <t>5014</t>
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>12015</v>
+        <v>6377</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>5023</t>
+          <t>5150</t>
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>6054</v>
+        <v>5381</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>5014</t>
+          <t>5170</t>
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>4669</v>
+        <v>4933</v>
       </c>
     </row>
     <row r="23">
@@ -5683,61 +5771,61 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>5150</t>
+          <t>5041</t>
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>4577</v>
+        <v>2197</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>5170</t>
+          <t>5011</t>
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>3644</v>
+        <v>1849</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>5041</t>
+          <t>5024</t>
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>2197</v>
+        <v>1520</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>5011</t>
+          <t>5120</t>
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>1331</v>
+        <v>769</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>5024</t>
+          <t>5210</t>
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>1137</v>
+        <v>733</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>5120</t>
+          <t>5004</t>
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>769</v>
+        <v>604</v>
       </c>
     </row>
     <row r="30">
@@ -5753,107 +5841,107 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>5210</t>
+          <t>5120</t>
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>485</v>
+        <v>355</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>5004</t>
+          <t>5300</t>
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>432</v>
+        <v>252</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>5120</t>
+          <t>5190</t>
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>355</v>
+        <v>238</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>5300</t>
+          <t>5070</t>
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>252</v>
+        <v>72</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>5190</t>
+          <t>5200</t>
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>192</v>
+        <v>66</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>5070</t>
+          <t>5180</t>
         </is>
       </c>
       <c r="B36" s="5" t="n">
-        <v>72</v>
+        <v>58</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>5180</t>
+          <t>5027</t>
         </is>
       </c>
       <c r="B37" s="5" t="n">
-        <v>44</v>
+        <v>29</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>5200</t>
+          <t>5250</t>
         </is>
       </c>
       <c r="B38" s="5" t="n">
-        <v>42</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>5027</t>
+          <t>5026</t>
         </is>
       </c>
       <c r="B39" s="5" t="n">
-        <v>21</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>5250</t>
+          <t>5220</t>
         </is>
       </c>
       <c r="B40" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>5026</t>
+          <t>5230</t>
         </is>
       </c>
       <c r="B41" s="5" t="n">
@@ -5863,7 +5951,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>5220</t>
+          <t>5260</t>
         </is>
       </c>
       <c r="B42" s="5" t="n">
@@ -5873,30 +5961,10 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>5230</t>
+          <t>5270</t>
         </is>
       </c>
       <c r="B43" s="5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>5260</t>
-        </is>
-      </c>
-      <c r="B44" s="5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>5270</t>
-        </is>
-      </c>
-      <c r="B45" s="5" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
AstraZeneca: cargar presupuesto integral Elegir Salud (no la línea de Avanter)
- AZ ahora refleja el presupuesto mensual completo (operación + call center +
  cápitas + auditorías + supervisor CS): ene 20.929.743,55 · feb 19.689.476,25 ·
  mar 21.612.629,37 · abr 21.786.516,13.
- Antes cargaba la línea de Avanter ($3-3,9M/mes), que subestimaba al cliente.
- Total general: $299.622.303,70 -> $370.153.282,00. AZ pasa a #2 (22,7%).
- Notas, fuentes y CLAUDE.md actualizados.
</commit_message>
<xml_diff>
--- a/Reporte_Labos_2026.xlsx
+++ b/Reporte_Labos_2026.xlsx
@@ -947,18 +947,18 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Uso plataforma MAT + TRX x valor unitario</t>
+          <t>Presupuesto Elegir Salud: operación + call center + cápitas + auditorías + supervisor CS</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Mensual por IPC Caba</t>
+          <t>Mensual por IPC CABA</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
@@ -973,10 +973,10 @@
         <v>0.0158272425784017</v>
       </c>
       <c r="L4" s="7" t="n">
-        <v>3164020</v>
+        <v>20929743.55</v>
       </c>
       <c r="M4" s="8" t="n">
-        <v>201.1455816910362</v>
+        <v>1330.562209154482</v>
       </c>
       <c r="N4" s="5" t="n">
         <v>13198</v>
@@ -985,10 +985,10 @@
         <v>0.01912191051038608</v>
       </c>
       <c r="P4" s="7" t="n">
-        <v>2976652</v>
+        <v>19689476.25</v>
       </c>
       <c r="Q4" s="8" t="n">
-        <v>225.5381118351265</v>
+        <v>1491.853026973784</v>
       </c>
       <c r="R4" s="5" t="n">
         <v>14775</v>
@@ -997,10 +997,10 @@
         <v>0.02184765346590287</v>
       </c>
       <c r="T4" s="7" t="n">
-        <v>3447758</v>
+        <v>21612629.37</v>
       </c>
       <c r="U4" s="8" t="n">
-        <v>233.3507952622674</v>
+        <v>1462.783713705584</v>
       </c>
       <c r="V4" s="5" t="n">
         <v>14849</v>
@@ -1009,10 +1009,10 @@
         <v>0.02303506219109996</v>
       </c>
       <c r="X4" s="7" t="n">
-        <v>3898957</v>
+        <v>21786516.13</v>
       </c>
       <c r="Y4" s="8" t="n">
-        <v>262.5737086672503</v>
+        <v>1467.204264933665</v>
       </c>
       <c r="BF4" s="9" t="n">
         <v>58552</v>
@@ -1021,10 +1021,10 @@
         <v>0.01948512442266267</v>
       </c>
       <c r="BH4" s="10" t="n">
-        <v>13487387</v>
+        <v>84018365.3</v>
       </c>
       <c r="BI4" s="8" t="n">
-        <v>230.348869381063</v>
+        <v>1434.935874094822</v>
       </c>
     </row>
     <row r="5">
@@ -5017,7 +5017,7 @@
       </c>
       <c r="K56" s="13" t="n"/>
       <c r="L56" s="14" t="n">
-        <v>88632610.45</v>
+        <v>106398334</v>
       </c>
       <c r="M56" s="13" t="n"/>
       <c r="N56" s="12" t="n">
@@ -5025,7 +5025,7 @@
       </c>
       <c r="O56" s="13" t="n"/>
       <c r="P56" s="14" t="n">
-        <v>64684069.98999999</v>
+        <v>81396894.23999999</v>
       </c>
       <c r="Q56" s="13" t="n"/>
       <c r="R56" s="12" t="n">
@@ -5033,7 +5033,7 @@
       </c>
       <c r="S56" s="13" t="n"/>
       <c r="T56" s="14" t="n">
-        <v>67359067</v>
+        <v>85523938.37</v>
       </c>
       <c r="U56" s="13" t="n"/>
       <c r="V56" s="12" t="n">
@@ -5041,7 +5041,7 @@
       </c>
       <c r="W56" s="13" t="n"/>
       <c r="X56" s="14" t="n">
-        <v>78946556.27</v>
+        <v>96834115.39999999</v>
       </c>
       <c r="Y56" s="13" t="n"/>
       <c r="Z56" s="12" t="n"/>
@@ -5081,7 +5081,7 @@
       </c>
       <c r="BG56" s="13" t="n"/>
       <c r="BH56" s="14" t="n">
-        <v>299622303.71</v>
+        <v>370153282.01</v>
       </c>
       <c r="BI56" s="13" t="n"/>
     </row>
@@ -5180,19 +5180,19 @@
         </is>
       </c>
       <c r="B4" s="8" t="n">
-        <v>203.33</v>
+        <v>360.85</v>
       </c>
       <c r="C4" s="8" t="n">
-        <v>198.11</v>
+        <v>360.96</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>194.3</v>
+        <v>320.51</v>
       </c>
       <c r="E4" s="8" t="n">
-        <v>201.34</v>
+        <v>315.69</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>199.17</v>
+        <v>335.92</v>
       </c>
     </row>
     <row r="5">
@@ -5251,7 +5251,7 @@
         <v>58552</v>
       </c>
       <c r="C9" s="7" t="n">
-        <v>13487387</v>
+        <v>84018365.3</v>
       </c>
     </row>
     <row r="10">
@@ -5505,7 +5505,7 @@
         </is>
       </c>
       <c r="B3" s="8" t="n">
-        <v>199.17</v>
+        <v>335.92</v>
       </c>
     </row>
     <row r="4">

</xml_diff>

<commit_message>
Completar meses faltantes desde planilla Seguimiento Facturación
- La planilla lista facturas por mes de EMISIÓN (servicio = mes anterior);
  cruzada así coincide al peso con el reporte en todos los clientes.
- Nuevos: Colgate feb 1.740.460 · Max Vision feb 1.188.815 · Health Care
  ene 971.876 y mar 904.782 · Lazar feb-mar 500.000 c/u · Sidus Farma feb
  131.941 · Ceoderma feb 0.
- Sidus Dermo abril corregido a 3.633.862,44 / 4.445 TRX (proforma + FC 370).
- Panalab queda solo fee/servicio (sin reintegro de bonos), confirmado.
- Total: 370.153.282,00 -> 377.426.332,29.
</commit_message>
<xml_diff>
--- a/Reporte_Labos_2026.xlsx
+++ b/Reporte_Labos_2026.xlsx
@@ -1006,7 +1006,7 @@
         <v>14849</v>
       </c>
       <c r="W4" s="6" t="n">
-        <v>0.02303506219109996</v>
+        <v>0.02305058119318464</v>
       </c>
       <c r="X4" s="7" t="n">
         <v>21786516.13</v>
@@ -1018,7 +1018,7 @@
         <v>58552</v>
       </c>
       <c r="BG4" s="6" t="n">
-        <v>0.01948512442266267</v>
+        <v>0.0194879390253035</v>
       </c>
       <c r="BH4" s="10" t="n">
         <v>84018365.3</v>
@@ -1116,7 +1116,7 @@
         <v>1178</v>
       </c>
       <c r="W6" s="6" t="n">
-        <v>0.001827416207227136</v>
+        <v>0.001828647359793354</v>
       </c>
       <c r="X6" s="7" t="n">
         <v>1075303.74</v>
@@ -1128,7 +1128,7 @@
         <v>4603</v>
       </c>
       <c r="BG6" s="6" t="n">
-        <v>0.001531801265840898</v>
+        <v>0.001532022532679874</v>
       </c>
       <c r="BH6" s="10" t="n">
         <v>4033286.55</v>
@@ -1223,28 +1223,28 @@
         <v>570.4299185597943</v>
       </c>
       <c r="V8" s="5" t="n">
-        <v>4879</v>
+        <v>4445</v>
       </c>
       <c r="W8" s="6" t="n">
-        <v>0.007568729775094396</v>
+        <v>0.00690011673538324</v>
       </c>
       <c r="X8" s="7" t="n">
-        <v>2298686.15</v>
+        <v>3633862.44</v>
       </c>
       <c r="Y8" s="8" t="n">
-        <v>471.1387886862062</v>
+        <v>817.516859392576</v>
       </c>
       <c r="BF8" s="9" t="n">
-        <v>12015</v>
+        <v>11581</v>
       </c>
       <c r="BG8" s="6" t="n">
-        <v>0.003998390660238625</v>
+        <v>0.003854519433188274</v>
       </c>
       <c r="BH8" s="10" t="n">
-        <v>6167887.15</v>
+        <v>7503063.44</v>
       </c>
       <c r="BI8" s="8" t="n">
-        <v>513.3489096962131</v>
+        <v>647.876991624212</v>
       </c>
     </row>
     <row r="9">
@@ -1301,6 +1301,9 @@
       <c r="M9" s="8" t="n">
         <v>1114.421031976744</v>
       </c>
+      <c r="P9" s="7" t="n">
+        <v>131941</v>
+      </c>
       <c r="R9" s="5" t="n">
         <v>615</v>
       </c>
@@ -1317,7 +1320,7 @@
         <v>894</v>
       </c>
       <c r="W9" s="6" t="n">
-        <v>0.0013868506700009</v>
+        <v>0.001387785008196314</v>
       </c>
       <c r="X9" s="7" t="n">
         <v>766721.67</v>
@@ -1329,13 +1332,13 @@
         <v>2197</v>
       </c>
       <c r="BG9" s="6" t="n">
-        <v>0.0007311247840652734</v>
+        <v>0.0007312303941554822</v>
       </c>
       <c r="BH9" s="10" t="n">
-        <v>2300165.01</v>
+        <v>2432106.01</v>
       </c>
       <c r="BI9" s="8" t="n">
-        <v>1046.957218934911</v>
+        <v>1107.012294037324</v>
       </c>
     </row>
     <row r="10">
@@ -1427,7 +1430,7 @@
         <v>4586</v>
       </c>
       <c r="W11" s="6" t="n">
-        <v>0.007114202653941975</v>
+        <v>0.007118995578957826</v>
       </c>
       <c r="X11" s="7" t="n">
         <v>9065584</v>
@@ -1439,7 +1442,7 @@
         <v>16933</v>
       </c>
       <c r="BG11" s="6" t="n">
-        <v>0.005635018647509001</v>
+        <v>0.005635832619132808</v>
       </c>
       <c r="BH11" s="10" t="n">
         <v>31379293</v>
@@ -1530,7 +1533,7 @@
         <v>103401</v>
       </c>
       <c r="W12" s="6" t="n">
-        <v>0.1604046377279228</v>
+        <v>0.1605127042869207</v>
       </c>
       <c r="X12" s="7" t="n">
         <v>10793227.5</v>
@@ -1542,7 +1545,7 @@
         <v>339671</v>
       </c>
       <c r="BG12" s="6" t="n">
-        <v>0.1130368168084823</v>
+        <v>0.1130531448398665</v>
       </c>
       <c r="BH12" s="10" t="n">
         <v>34846389.1</v>
@@ -1612,6 +1615,9 @@
       <c r="M14" s="8" t="n">
         <v>95.45023500855078</v>
       </c>
+      <c r="P14" s="7" t="n">
+        <v>1740460</v>
+      </c>
       <c r="R14" s="5" t="n">
         <v>23875</v>
       </c>
@@ -1628,7 +1634,7 @@
         <v>20351</v>
       </c>
       <c r="W14" s="6" t="n">
-        <v>0.03157024383130683</v>
+        <v>0.03159151308926531</v>
       </c>
       <c r="X14" s="7" t="n">
         <v>1876522.43</v>
@@ -1640,13 +1646,13 @@
         <v>62353</v>
       </c>
       <c r="BG14" s="6" t="n">
-        <v>0.02075003352791169</v>
+        <v>0.02075303084514191</v>
       </c>
       <c r="BH14" s="10" t="n">
-        <v>5945633.78</v>
+        <v>7686093.78</v>
       </c>
       <c r="BI14" s="8" t="n">
-        <v>95.35441406187351</v>
+        <v>123.2674254646929</v>
       </c>
     </row>
     <row r="15">
@@ -1710,6 +1716,9 @@
       <c r="M16" s="8" t="n">
         <v>208.161474084641</v>
       </c>
+      <c r="P16" s="7" t="n">
+        <v>1188815</v>
+      </c>
       <c r="R16" s="5" t="n">
         <v>6019</v>
       </c>
@@ -1726,7 +1735,7 @@
         <v>6040</v>
       </c>
       <c r="W16" s="6" t="n">
-        <v>0.009369774101572075</v>
+        <v>0.009376086632556754</v>
       </c>
       <c r="X16" s="7" t="n">
         <v>1378201.65</v>
@@ -1738,13 +1747,13 @@
         <v>18368</v>
       </c>
       <c r="BG16" s="6" t="n">
-        <v>0.00611256260068773</v>
+        <v>0.006113445552957622</v>
       </c>
       <c r="BH16" s="10" t="n">
-        <v>4059529.29</v>
+        <v>5248344.29</v>
       </c>
       <c r="BI16" s="8" t="n">
-        <v>221.0109587325784</v>
+        <v>285.7330297256097</v>
       </c>
     </row>
     <row r="17">
@@ -1836,7 +1845,7 @@
         <v>9</v>
       </c>
       <c r="W18" s="6" t="n">
-        <v>1.396158392618356e-05</v>
+        <v>1.397099001539914e-05</v>
       </c>
       <c r="X18" s="7" t="n">
         <v>837</v>
@@ -1848,7 +1857,7 @@
         <v>72</v>
       </c>
       <c r="BG18" s="6" t="n">
-        <v>2.396039346959476e-05</v>
+        <v>2.396385451943319e-05</v>
       </c>
       <c r="BH18" s="10" t="n">
         <v>5499</v>
@@ -1918,11 +1927,14 @@
       <c r="M20" s="8" t="n">
         <v>207.8091027308193</v>
       </c>
+      <c r="P20" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="BF20" s="9" t="n">
         <v>769</v>
       </c>
       <c r="BG20" s="6" t="n">
-        <v>0.0002559103135849774</v>
+        <v>0.0002559472795200572</v>
       </c>
       <c r="BH20" s="10" t="n">
         <v>159805.2</v>
@@ -1980,14 +1992,20 @@
           <t>PRODUCTIVO</t>
         </is>
       </c>
+      <c r="L22" s="7" t="n">
+        <v>971876</v>
+      </c>
       <c r="P22" s="7" t="n">
         <v>871875.5</v>
       </c>
+      <c r="T22" s="7" t="n">
+        <v>904782</v>
+      </c>
       <c r="X22" s="7" t="n">
         <v>952203.02</v>
       </c>
       <c r="BH22" s="10" t="n">
-        <v>1824078.52</v>
+        <v>3700736.52</v>
       </c>
     </row>
     <row r="23">
@@ -2042,11 +2060,17 @@
       <c r="L24" s="7" t="n">
         <v>500000</v>
       </c>
+      <c r="P24" s="7" t="n">
+        <v>500000</v>
+      </c>
+      <c r="T24" s="7" t="n">
+        <v>500000</v>
+      </c>
       <c r="V24" s="5" t="n">
         <v>252</v>
       </c>
       <c r="W24" s="6" t="n">
-        <v>0.0003909243499331395</v>
+        <v>0.0003911877204311758</v>
       </c>
       <c r="X24" s="7" t="n">
         <v>344079.51</v>
@@ -2058,13 +2082,13 @@
         <v>252</v>
       </c>
       <c r="BG24" s="6" t="n">
-        <v>8.386137714358165e-05</v>
+        <v>8.387349081801616e-05</v>
       </c>
       <c r="BH24" s="10" t="n">
-        <v>844079.51</v>
+        <v>1844079.51</v>
       </c>
       <c r="BI24" s="8" t="n">
-        <v>3349.521865079365</v>
+        <v>7317.775833333333</v>
       </c>
     </row>
     <row r="25">
@@ -2160,7 +2184,7 @@
         <v>150</v>
       </c>
       <c r="W26" s="6" t="n">
-        <v>0.0002326930654363926</v>
+        <v>0.0002328498335899856</v>
       </c>
       <c r="X26" s="7" t="n">
         <v>13950</v>
@@ -2172,7 +2196,7 @@
         <v>604</v>
       </c>
       <c r="BG26" s="6" t="n">
-        <v>0.0002010010785504894</v>
+        <v>0.0002010301129130229</v>
       </c>
       <c r="BH26" s="10" t="n">
         <v>47546</v>
@@ -2267,7 +2291,7 @@
         <v>67206</v>
       </c>
       <c r="W27" s="6" t="n">
-        <v>0.1042558010381213</v>
+        <v>0.1043260394416572</v>
       </c>
       <c r="X27" s="7" t="n">
         <v>6250158</v>
@@ -2279,7 +2303,7 @@
         <v>308616</v>
       </c>
       <c r="BG27" s="6" t="n">
-        <v>0.1027022332085063</v>
+        <v>0.1027170684217971</v>
       </c>
       <c r="BH27" s="10" t="n">
         <v>24114498</v>
@@ -2374,7 +2398,7 @@
         <v>484</v>
       </c>
       <c r="W28" s="6" t="n">
-        <v>0.0007508229578080934</v>
+        <v>0.0007513287963836869</v>
       </c>
       <c r="X28" s="7" t="n">
         <v>45012</v>
@@ -2386,7 +2410,7 @@
         <v>1849</v>
       </c>
       <c r="BG28" s="6" t="n">
-        <v>0.0006153162156288987</v>
+        <v>0.000615405097311555</v>
       </c>
       <c r="BH28" s="10" t="n">
         <v>146022</v>
@@ -2481,7 +2505,7 @@
         <v>1683</v>
       </c>
       <c r="W29" s="6" t="n">
-        <v>0.002610816194196325</v>
+        <v>0.002612575132879639</v>
       </c>
       <c r="X29" s="7" t="n">
         <v>156519</v>
@@ -2493,7 +2517,7 @@
         <v>6377</v>
       </c>
       <c r="BG29" s="6" t="n">
-        <v>0.002122158738272303</v>
+        <v>0.002122465281533687</v>
       </c>
       <c r="BH29" s="10" t="n">
         <v>503875</v>
@@ -2588,7 +2612,7 @@
         <v>29074</v>
       </c>
       <c r="W30" s="6" t="n">
-        <v>0.04510212122998452</v>
+        <v>0.04513250707863494</v>
       </c>
       <c r="X30" s="7" t="n">
         <v>2703882</v>
@@ -2600,7 +2624,7 @@
         <v>136340</v>
       </c>
       <c r="BG30" s="6" t="n">
-        <v>0.04537166730061874</v>
+        <v>0.0453782211830489</v>
       </c>
       <c r="BH30" s="10" t="n">
         <v>10641566</v>
@@ -2695,7 +2719,7 @@
         <v>25273</v>
       </c>
       <c r="W31" s="6" t="n">
-        <v>0.03920567895182633</v>
+        <v>0.0392320922954647</v>
       </c>
       <c r="X31" s="7" t="n">
         <v>2350389</v>
@@ -2707,7 +2731,7 @@
         <v>116927</v>
       </c>
       <c r="BG31" s="6" t="n">
-        <v>0.03891134621137925</v>
+        <v>0.03891696690824673</v>
       </c>
       <c r="BH31" s="10" t="n">
         <v>9132785</v>
@@ -2802,7 +2826,7 @@
         <v>2285</v>
       </c>
       <c r="W32" s="6" t="n">
-        <v>0.003544691030147714</v>
+        <v>0.003547079131687447</v>
       </c>
       <c r="X32" s="7" t="n">
         <v>212505</v>
@@ -2814,7 +2838,7 @@
         <v>8151</v>
       </c>
       <c r="BG32" s="6" t="n">
-        <v>0.002712516210703707</v>
+        <v>0.002712908030387499</v>
       </c>
       <c r="BH32" s="10" t="n">
         <v>646589</v>
@@ -2909,7 +2933,7 @@
         <v>421</v>
       </c>
       <c r="W33" s="6" t="n">
-        <v>0.0006530918703248085</v>
+        <v>0.0006535318662758929</v>
       </c>
       <c r="X33" s="7" t="n">
         <v>39153</v>
@@ -2921,7 +2945,7 @@
         <v>1520</v>
       </c>
       <c r="BG33" s="6" t="n">
-        <v>0.0005058305288025561</v>
+        <v>0.0005059035954102562</v>
       </c>
       <c r="BH33" s="10" t="n">
         <v>120479</v>
@@ -3016,7 +3040,7 @@
         <v>8</v>
       </c>
       <c r="W34" s="6" t="n">
-        <v>1.241029682327427e-05</v>
+        <v>1.24186577914659e-05</v>
       </c>
       <c r="X34" s="7" t="n">
         <v>744</v>
@@ -3028,7 +3052,7 @@
         <v>29</v>
       </c>
       <c r="BG34" s="6" t="n">
-        <v>9.650714036364556e-06</v>
+        <v>9.652108070327256e-06</v>
       </c>
       <c r="BH34" s="10" t="n">
         <v>2298</v>
@@ -3123,7 +3147,7 @@
         <v>260641</v>
       </c>
       <c r="W35" s="6" t="n">
-        <v>0.4043290217893786</v>
+        <v>0.4046014231781829</v>
       </c>
       <c r="X35" s="7" t="n">
         <v>24239613</v>
@@ -3135,7 +3159,7 @@
         <v>1425880</v>
       </c>
       <c r="BG35" s="6" t="n">
-        <v>0.4745089700059136</v>
+        <v>0.4745775122523527</v>
       </c>
       <c r="BH35" s="10" t="n">
         <v>110467299</v>
@@ -3230,7 +3254,7 @@
         <v>18937</v>
       </c>
       <c r="W36" s="6" t="n">
-        <v>0.02937672386779311</v>
+        <v>0.02939651532462371</v>
       </c>
       <c r="X36" s="7" t="n">
         <v>1761141</v>
@@ -3242,7 +3266,7 @@
         <v>105857</v>
       </c>
       <c r="BG36" s="6" t="n">
-        <v>0.03522743571542906</v>
+        <v>0.03523252427588387</v>
       </c>
       <c r="BH36" s="10" t="n">
         <v>8193221</v>
@@ -3337,7 +3361,7 @@
         <v>9934</v>
       </c>
       <c r="W37" s="6" t="n">
-        <v>0.01541048608030083</v>
+        <v>0.01542086831255278</v>
       </c>
       <c r="X37" s="7" t="n">
         <v>923862</v>
@@ -3349,7 +3373,7 @@
         <v>38929</v>
       </c>
       <c r="BG37" s="6" t="n">
-        <v>0.0129549188524702</v>
+        <v>0.01295679017481965</v>
       </c>
       <c r="BH37" s="10" t="n">
         <v>3069492</v>
@@ -3444,7 +3468,7 @@
         <v>4464</v>
       </c>
       <c r="W38" s="6" t="n">
-        <v>0.006924945627387043</v>
+        <v>0.006929611047637971</v>
       </c>
       <c r="X38" s="7" t="n">
         <v>415152</v>
@@ -3456,7 +3480,7 @@
         <v>17738</v>
       </c>
       <c r="BG38" s="6" t="n">
-        <v>0.005902909157828776</v>
+        <v>0.005903761825912582</v>
       </c>
       <c r="BH38" s="10" t="n">
         <v>1397428</v>
@@ -3551,7 +3575,7 @@
         <v>31434</v>
       </c>
       <c r="W39" s="6" t="n">
-        <v>0.04876315879285043</v>
+        <v>0.04879601112711738</v>
       </c>
       <c r="X39" s="7" t="n">
         <v>2923362</v>
@@ -3563,7 +3587,7 @@
         <v>113488</v>
       </c>
       <c r="BG39" s="6" t="n">
-        <v>0.03776690463996348</v>
+        <v>0.03777236002363103</v>
       </c>
       <c r="BH39" s="10" t="n">
         <v>8995358</v>
@@ -3634,7 +3658,7 @@
         <v>355</v>
       </c>
       <c r="BG40" s="6" t="n">
-        <v>0.0001181380511348075</v>
+        <v>0.0001181551160333164</v>
       </c>
       <c r="BH40" s="10" t="n">
         <v>26270</v>
@@ -3729,7 +3753,7 @@
         <v>9823</v>
       </c>
       <c r="W41" s="6" t="n">
-        <v>0.0152382932118779</v>
+        <v>0.01524855943569619</v>
       </c>
       <c r="X41" s="7" t="n">
         <v>913539</v>
@@ -3741,7 +3765,7 @@
         <v>36047</v>
       </c>
       <c r="BG41" s="6" t="n">
-        <v>0.01199583754720114</v>
+        <v>0.01199757033141678</v>
       </c>
       <c r="BH41" s="10" t="n">
         <v>2854115</v>
@@ -3836,7 +3860,7 @@
         <v>15759</v>
       </c>
       <c r="W42" s="6" t="n">
-        <v>0.0244467334547474</v>
+        <v>0.02446320351696389</v>
       </c>
       <c r="X42" s="7" t="n">
         <v>1465587</v>
@@ -3848,7 +3872,7 @@
         <v>135617</v>
       </c>
       <c r="BG42" s="6" t="n">
-        <v>0.0451310650161949</v>
+        <v>0.04513758414391626</v>
       </c>
       <c r="BH42" s="10" t="n">
         <v>10335079</v>
@@ -3943,7 +3967,7 @@
         <v>2593</v>
       </c>
       <c r="W43" s="6" t="n">
-        <v>0.004022487457843773</v>
+        <v>0.004025197456658885</v>
       </c>
       <c r="X43" s="7" t="n">
         <v>241149</v>
@@ -3955,7 +3979,7 @@
         <v>5381</v>
       </c>
       <c r="BG43" s="6" t="n">
-        <v>0.001790706628609575</v>
+        <v>0.001790965294014861</v>
       </c>
       <c r="BH43" s="10" t="n">
         <v>447461</v>
@@ -4050,7 +4074,7 @@
         <v>6100</v>
       </c>
       <c r="W44" s="6" t="n">
-        <v>0.009462851327746631</v>
+        <v>0.009469226565992748</v>
       </c>
       <c r="X44" s="7" t="n">
         <v>567300</v>
@@ -4062,7 +4086,7 @@
         <v>22917</v>
       </c>
       <c r="BG44" s="6" t="n">
-        <v>0.007626393571426432</v>
+        <v>0.007627495194747922</v>
       </c>
       <c r="BH44" s="10" t="n">
         <v>1811758</v>
@@ -4157,7 +4181,7 @@
         <v>1462</v>
       </c>
       <c r="W45" s="6" t="n">
-        <v>0.002267981744453373</v>
+        <v>0.002269509711390393</v>
       </c>
       <c r="X45" s="7" t="n">
         <v>135966</v>
@@ -4169,7 +4193,7 @@
         <v>4933</v>
       </c>
       <c r="BG45" s="6" t="n">
-        <v>0.001641619735909874</v>
+        <v>0.001641856865893943</v>
       </c>
       <c r="BH45" s="10" t="n">
         <v>392820</v>
@@ -4264,7 +4288,7 @@
         <v>22</v>
       </c>
       <c r="W46" s="6" t="n">
-        <v>3.412831626400425e-05</v>
+        <v>3.415130892653122e-05</v>
       </c>
       <c r="X46" s="7" t="n">
         <v>2046</v>
@@ -4276,7 +4300,7 @@
         <v>58</v>
       </c>
       <c r="BG46" s="6" t="n">
-        <v>1.930142807272911e-05</v>
+        <v>1.930421614065451e-05</v>
       </c>
       <c r="BH46" s="10" t="n">
         <v>4710</v>
@@ -4371,7 +4395,7 @@
         <v>107</v>
       </c>
       <c r="W47" s="6" t="n">
-        <v>0.0001659877200112934</v>
+        <v>0.0001660995479608564</v>
       </c>
       <c r="X47" s="7" t="n">
         <v>9951</v>
@@ -4383,7 +4407,7 @@
         <v>238</v>
       </c>
       <c r="BG47" s="6" t="n">
-        <v>7.920241174671601e-05</v>
+        <v>7.921385243923749e-05</v>
       </c>
       <c r="BH47" s="10" t="n">
         <v>19645</v>
@@ -4478,7 +4502,7 @@
         <v>6</v>
       </c>
       <c r="W48" s="6" t="n">
-        <v>9.307722617455703e-06</v>
+        <v>9.313993343599423e-06</v>
       </c>
       <c r="X48" s="7" t="n">
         <v>558</v>
@@ -4490,7 +4514,7 @@
         <v>66</v>
       </c>
       <c r="BG48" s="6" t="n">
-        <v>2.19636940137952e-05</v>
+        <v>2.196686664281376e-05</v>
       </c>
       <c r="BH48" s="10" t="n">
         <v>4998</v>
@@ -4585,7 +4609,7 @@
         <v>320</v>
       </c>
       <c r="W49" s="6" t="n">
-        <v>0.0004964118729309709</v>
+        <v>0.0004967463116586359</v>
       </c>
       <c r="X49" s="7" t="n">
         <v>29760</v>
@@ -4597,7 +4621,7 @@
         <v>733</v>
       </c>
       <c r="BG49" s="6" t="n">
-        <v>0.00024393011685018</v>
+        <v>0.0002439653522603406</v>
       </c>
       <c r="BH49" s="10" t="n">
         <v>60322</v>
@@ -4810,7 +4834,7 @@
         <v>523</v>
       </c>
       <c r="BG52" s="6" t="n">
-        <v>0.0001740456358971953</v>
+        <v>0.0001740707765786605</v>
       </c>
       <c r="BH52" s="10" t="n">
         <v>38702</v>
@@ -4887,7 +4911,7 @@
         <v>1</v>
       </c>
       <c r="W53" s="6" t="n">
-        <v>1.551287102909284e-06</v>
+        <v>1.552332223933237e-06</v>
       </c>
       <c r="X53" s="7" t="n">
         <v>93</v>
@@ -4899,7 +4923,7 @@
         <v>1</v>
       </c>
       <c r="BG53" s="6" t="n">
-        <v>3.327832426332606e-07</v>
+        <v>3.328313127699054e-07</v>
       </c>
       <c r="BH53" s="10" t="n">
         <v>93</v>
@@ -5017,7 +5041,7 @@
       </c>
       <c r="K56" s="13" t="n"/>
       <c r="L56" s="14" t="n">
-        <v>106398334</v>
+        <v>107370210</v>
       </c>
       <c r="M56" s="13" t="n"/>
       <c r="N56" s="12" t="n">
@@ -5025,7 +5049,7 @@
       </c>
       <c r="O56" s="13" t="n"/>
       <c r="P56" s="14" t="n">
-        <v>81396894.23999999</v>
+        <v>84958110.23999999</v>
       </c>
       <c r="Q56" s="13" t="n"/>
       <c r="R56" s="12" t="n">
@@ -5033,15 +5057,15 @@
       </c>
       <c r="S56" s="13" t="n"/>
       <c r="T56" s="14" t="n">
-        <v>85523938.37</v>
+        <v>86928720.37</v>
       </c>
       <c r="U56" s="13" t="n"/>
       <c r="V56" s="12" t="n">
-        <v>644626</v>
+        <v>644192</v>
       </c>
       <c r="W56" s="13" t="n"/>
       <c r="X56" s="14" t="n">
-        <v>96834115.39999999</v>
+        <v>98169291.69</v>
       </c>
       <c r="Y56" s="13" t="n"/>
       <c r="Z56" s="12" t="n"/>
@@ -5077,11 +5101,11 @@
       <c r="BD56" s="14" t="n"/>
       <c r="BE56" s="13" t="n"/>
       <c r="BF56" s="12" t="n">
-        <v>3004959</v>
+        <v>3004525</v>
       </c>
       <c r="BG56" s="13" t="n"/>
       <c r="BH56" s="14" t="n">
-        <v>370153282.01</v>
+        <v>377426332.3</v>
       </c>
       <c r="BI56" s="13" t="n"/>
     </row>
@@ -5189,10 +5213,10 @@
         <v>320.51</v>
       </c>
       <c r="E4" s="8" t="n">
-        <v>315.69</v>
+        <v>325.12</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>335.92</v>
+        <v>338.79</v>
       </c>
     </row>
     <row r="5">
@@ -5274,10 +5298,10 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>14212</v>
+        <v>13778</v>
       </c>
       <c r="C11" s="7" t="n">
-        <v>8468052.16</v>
+        <v>9935169.449999999</v>
       </c>
     </row>
     <row r="12">
@@ -5303,7 +5327,7 @@
         <v>62353</v>
       </c>
       <c r="C13" s="7" t="n">
-        <v>5945633.78</v>
+        <v>7686093.78</v>
       </c>
     </row>
     <row r="14">
@@ -5316,7 +5340,7 @@
         <v>18368</v>
       </c>
       <c r="C14" s="7" t="n">
-        <v>4059529.29</v>
+        <v>5248344.29</v>
       </c>
     </row>
     <row r="15">
@@ -5355,7 +5379,7 @@
         <v>0</v>
       </c>
       <c r="C17" s="7" t="n">
-        <v>1824078.52</v>
+        <v>3700736.52</v>
       </c>
     </row>
     <row r="18">
@@ -5368,7 +5392,7 @@
         <v>252</v>
       </c>
       <c r="C18" s="7" t="n">
-        <v>844079.51</v>
+        <v>1844079.51</v>
       </c>
     </row>
     <row r="19">
@@ -5505,7 +5529,7 @@
         </is>
       </c>
       <c r="B3" s="8" t="n">
-        <v>335.92</v>
+        <v>338.79</v>
       </c>
     </row>
     <row r="4">
@@ -5715,7 +5739,7 @@
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>12015</v>
+        <v>11581</v>
       </c>
     </row>
     <row r="19">

</xml_diff>

<commit_message>
BIU = Unyc S.A.: corregir montos reales de facturación; Iqvia excluido (pago anual)
- BIU (razón social Unyc S.A.) pasa de placeholder TRX*VU ($5.499) a la
  facturación real de la planilla: ene 9.033 / feb 7.296 / mar 8.322 / abr 3.404.
- Iqvia Solutions excluido del reporte por ser pago anual (no bonos mensuales);
  aclarado en notas.
- Total: 377.426.332,29 -> 377.448.888,29.
</commit_message>
<xml_diff>
--- a/Reporte_Labos_2026.xlsx
+++ b/Reporte_Labos_2026.xlsx
@@ -1771,7 +1771,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Bonos BIU Cosmeceuticals</t>
+          <t>Bonos BIU Cosmeceuticals (Unyc S.A.)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1812,10 +1812,10 @@
         <v>2.213600360615622e-05</v>
       </c>
       <c r="L18" s="7" t="n">
-        <v>1628</v>
+        <v>9033</v>
       </c>
       <c r="M18" s="8" t="n">
-        <v>74</v>
+        <v>410.5909090909091</v>
       </c>
       <c r="N18" s="5" t="n">
         <v>20</v>
@@ -1824,10 +1824,10 @@
         <v>2.897698213424167e-05</v>
       </c>
       <c r="P18" s="7" t="n">
-        <v>1480</v>
+        <v>7296</v>
       </c>
       <c r="Q18" s="8" t="n">
-        <v>74</v>
+        <v>364.8</v>
       </c>
       <c r="R18" s="5" t="n">
         <v>21</v>
@@ -1836,10 +1836,10 @@
         <v>3.10525023880853e-05</v>
       </c>
       <c r="T18" s="7" t="n">
-        <v>1554</v>
+        <v>8322</v>
       </c>
       <c r="U18" s="8" t="n">
-        <v>74</v>
+        <v>396.2857142857143</v>
       </c>
       <c r="V18" s="5" t="n">
         <v>9</v>
@@ -1848,10 +1848,10 @@
         <v>1.397099001539914e-05</v>
       </c>
       <c r="X18" s="7" t="n">
-        <v>837</v>
+        <v>3404</v>
       </c>
       <c r="Y18" s="8" t="n">
-        <v>93</v>
+        <v>378.2222222222222</v>
       </c>
       <c r="BF18" s="9" t="n">
         <v>72</v>
@@ -1860,10 +1860,10 @@
         <v>2.396385451943319e-05</v>
       </c>
       <c r="BH18" s="10" t="n">
-        <v>5499</v>
+        <v>28055</v>
       </c>
       <c r="BI18" s="8" t="n">
-        <v>76.375</v>
+        <v>389.6527777777778</v>
       </c>
     </row>
     <row r="19">
@@ -5041,7 +5041,7 @@
       </c>
       <c r="K56" s="13" t="n"/>
       <c r="L56" s="14" t="n">
-        <v>107370210</v>
+        <v>107377615</v>
       </c>
       <c r="M56" s="13" t="n"/>
       <c r="N56" s="12" t="n">
@@ -5049,7 +5049,7 @@
       </c>
       <c r="O56" s="13" t="n"/>
       <c r="P56" s="14" t="n">
-        <v>84958110.23999999</v>
+        <v>84963926.23999999</v>
       </c>
       <c r="Q56" s="13" t="n"/>
       <c r="R56" s="12" t="n">
@@ -5057,7 +5057,7 @@
       </c>
       <c r="S56" s="13" t="n"/>
       <c r="T56" s="14" t="n">
-        <v>86928720.37</v>
+        <v>86935488.37</v>
       </c>
       <c r="U56" s="13" t="n"/>
       <c r="V56" s="12" t="n">
@@ -5065,7 +5065,7 @@
       </c>
       <c r="W56" s="13" t="n"/>
       <c r="X56" s="14" t="n">
-        <v>98169291.69</v>
+        <v>98171858.69</v>
       </c>
       <c r="Y56" s="13" t="n"/>
       <c r="Z56" s="12" t="n"/>
@@ -5105,7 +5105,7 @@
       </c>
       <c r="BG56" s="13" t="n"/>
       <c r="BH56" s="14" t="n">
-        <v>377426332.3</v>
+        <v>377448888.3</v>
       </c>
       <c r="BI56" s="13" t="n"/>
     </row>
@@ -5204,19 +5204,19 @@
         </is>
       </c>
       <c r="B4" s="8" t="n">
-        <v>360.85</v>
+        <v>360.91</v>
       </c>
       <c r="C4" s="8" t="n">
-        <v>360.96</v>
+        <v>361.01</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>320.51</v>
+        <v>320.56</v>
       </c>
       <c r="E4" s="8" t="n">
-        <v>325.12</v>
+        <v>325.14</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>338.79</v>
+        <v>338.83</v>
       </c>
     </row>
     <row r="5">
@@ -5353,7 +5353,7 @@
         <v>72</v>
       </c>
       <c r="C15" s="7" t="n">
-        <v>5499</v>
+        <v>28055</v>
       </c>
     </row>
     <row r="16">
@@ -5529,7 +5529,7 @@
         </is>
       </c>
       <c r="B3" s="8" t="n">
-        <v>338.79</v>
+        <v>338.83</v>
       </c>
     </row>
     <row r="4">

</xml_diff>